<commit_message>
Rename enemy IDs and remove glossary sheets from game data
</commit_message>
<xml_diff>
--- a/docs/Dealbreak_GameData.xlsx
+++ b/docs/Dealbreak_GameData.xlsx
@@ -2,18 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="1" r:id="R42bdacdccd684fc9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bosses" sheetId="2" r:id="Rf912b4b6935e41c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gear" sheetId="3" r:id="R5825b6b43fe34e78"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enhancements" sheetId="4" r:id="R5a75b15a866a45bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Events" sheetId="5" r:id="R394592f3578c4cd8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shops" sheetId="6" r:id="Ra0364a62b4d94f4d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maps" sheetId="7" r:id="R761c735c31294c7d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consumables" sheetId="8" r:id="Rc38043941b004b0c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Boss Abilities" sheetId="9" r:id="Rb58408a2e69d4d01"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scaling" sheetId="10" r:id="R322d02a99b0446b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dealbreak Guide" sheetId="11" r:id="R49d3c9c8fc25486e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rename Index" sheetId="12" r:id="Re2d14e1db7d44fb2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="1" r:id="R5989d53704934f69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bosses" sheetId="2" r:id="R8449d58dc9584c1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gear" sheetId="3" r:id="R5290c2d27f364e89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enhancements" sheetId="4" r:id="R0b4a18f9a115498b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Events" sheetId="5" r:id="R24a5a13a648747a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shops" sheetId="6" r:id="Rcfe5520cf3c64426"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maps" sheetId="7" r:id="R0fc7a584066f4141"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consumables" sheetId="8" r:id="R1ab1407a85634dd7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Boss Abilities" sheetId="9" r:id="R7582c6e035704d42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scaling" sheetId="10" r:id="Rb11b081c26ad4b73"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -28,7 +26,7 @@
     <x:numFmt numFmtId="200" formatCode="0"/>
     <x:numFmt numFmtId="201" formatCode="0.00"/>
   </x:numFmts>
-  <x:fonts count="6">
+  <x:fonts count="3">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -44,26 +42,8 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Arial"/>
     </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="15"/>
-      <x:color rgb="FF202833"/>
-      <x:name val="Arial"/>
-    </x:font>
-    <x:font>
-      <x:i/>
-      <x:sz val="10"/>
-      <x:color rgb="FF4B5563"/>
-      <x:name val="Arial"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="11"/>
-      <x:color rgb="FF202833"/>
-      <x:name val="Arial"/>
-    </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="3">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -73,11 +53,6 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF1F2937"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFE5E7EB"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -93,7 +68,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="23">
+  <x:cellXfs count="19">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -147,43 +122,11 @@
     <x:xf numFmtId="201" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="22">
-    <x:dxf>
-      <x:font>
-        <x:color rgb="FF805500"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFFF0C2"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:color rgb="FF9B1C1C"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFDE2E2"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
+  <x:dxfs count="20">
     <x:dxf>
       <x:font>
         <x:color rgb="FF805500"/>
@@ -840,7 +783,7 @@
     </x:row>
     <x:row r="2" ht="55" customHeight="1">
       <x:c r="A2" s="3" t="str">
-        <x:v>foe_goblin</x:v>
+        <x:v>foe_scrapper</x:v>
       </x:c>
       <x:c r="B2" s="3" t="str">
         <x:v>Scrapper</x:v>
@@ -878,7 +821,7 @@
     </x:row>
     <x:row r="3" ht="40" customHeight="1">
       <x:c r="A3" s="3" t="str">
-        <x:v>foe_thief</x:v>
+        <x:v>foe_pickpocket</x:v>
       </x:c>
       <x:c r="B3" s="3" t="str">
         <x:v>Pickpocket</x:v>
@@ -916,7 +859,7 @@
     </x:row>
     <x:row r="4" ht="70" customHeight="1">
       <x:c r="A4" s="3" t="str">
-        <x:v>foe_knight</x:v>
+        <x:v>foe_security_guard</x:v>
       </x:c>
       <x:c r="B4" s="3" t="str">
         <x:v>Security Guard</x:v>
@@ -954,7 +897,7 @@
     </x:row>
     <x:row r="5" ht="55" customHeight="1">
       <x:c r="A5" s="3" t="str">
-        <x:v>foe_brute</x:v>
+        <x:v>foe_heavy</x:v>
       </x:c>
       <x:c r="B5" s="3" t="str">
         <x:v>Heavy</x:v>
@@ -992,7 +935,7 @@
     </x:row>
     <x:row r="6" ht="40" customHeight="1">
       <x:c r="A6" s="3" t="str">
-        <x:v>foe_shieldbearer</x:v>
+        <x:v>foe_riot_guard</x:v>
       </x:c>
       <x:c r="B6" s="3" t="str">
         <x:v>Riot Guard</x:v>
@@ -1030,7 +973,7 @@
     </x:row>
     <x:row r="7" ht="85" customHeight="1">
       <x:c r="A7" s="3" t="str">
-        <x:v>foe_war_drummer</x:v>
+        <x:v>foe_hype_man</x:v>
       </x:c>
       <x:c r="B7" s="3" t="str">
         <x:v>Hype Man</x:v>
@@ -1068,7 +1011,7 @@
     </x:row>
     <x:row r="8" ht="40" customHeight="1">
       <x:c r="A8" s="3" t="str">
-        <x:v>foe_duelist</x:v>
+        <x:v>foe_challenger</x:v>
       </x:c>
       <x:c r="B8" s="3" t="str">
         <x:v>Challenger</x:v>
@@ -1106,7 +1049,7 @@
     </x:row>
     <x:row r="9" ht="70" customHeight="1">
       <x:c r="A9" s="3" t="str">
-        <x:v>foe_goblin_captain</x:v>
+        <x:v>foe_crew_leader</x:v>
       </x:c>
       <x:c r="B9" s="3" t="str">
         <x:v>Crew Leader</x:v>
@@ -1144,7 +1087,7 @@
     </x:row>
     <x:row r="10" ht="55" customHeight="1">
       <x:c r="A10" s="3" t="str">
-        <x:v>foe_royal_knight</x:v>
+        <x:v>foe_riot_captain</x:v>
       </x:c>
       <x:c r="B10" s="3" t="str">
         <x:v>Riot Captain</x:v>
@@ -1182,7 +1125,7 @@
     </x:row>
     <x:row r="11" ht="100" customHeight="1">
       <x:c r="A11" s="3" t="str">
-        <x:v>foe_master_thief</x:v>
+        <x:v>foe_ghost</x:v>
       </x:c>
       <x:c r="B11" s="3" t="str">
         <x:v>Ghost</x:v>
@@ -1230,7 +1173,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R948158838ba14f8f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80095c9d0f024d86"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1530,4299 +1473,8 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf58d6ffe637d4761"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R533d0e2604754346"/>
   </x:tableParts>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="29" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="29" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="29" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="68" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="31" customHeight="1">
-      <x:c r="A1" s="19" t="str">
-        <x:v>DEALBREAK  /  GAME DATA LANGUAGE</x:v>
-      </x:c>
-      <x:c r="B1" s="3"/>
-      <x:c r="C1" s="3"/>
-      <x:c r="D1" s="3"/>
-      <x:c r="E1" s="3"/>
-    </x:row>
-    <x:row r="2" ht="35" customHeight="1">
-      <x:c r="A2" s="20" t="str">
-        <x:v>A modern, underground, slightly surreal card roguelike — not medieval fantasy.</x:v>
-      </x:c>
-      <x:c r="B2" s="3"/>
-      <x:c r="C2" s="3"/>
-      <x:c r="D2" s="3"/>
-      <x:c r="E2" s="3"/>
-    </x:row>
-    <x:row r="3" ht="24" customHeight="1">
-      <x:c r="A3" s="3"/>
-      <x:c r="B3" s="3"/>
-      <x:c r="C3" s="3"/>
-      <x:c r="D3" s="3"/>
-      <x:c r="E3" s="3"/>
-    </x:row>
-    <x:row r="4" ht="28" customHeight="1">
-      <x:c r="A4" s="22" t="str">
-        <x:v>CANONICAL PLAYER-FACING TERMINOLOGY</x:v>
-      </x:c>
-      <x:c r="B4" s="22"/>
-      <x:c r="C4" s="22"/>
-      <x:c r="D4" s="22"/>
-      <x:c r="E4" s="22"/>
-    </x:row>
-    <x:row r="5" ht="38" customHeight="1">
-      <x:c r="A5" s="12" t="str">
-        <x:v>Context</x:v>
-      </x:c>
-      <x:c r="B5" s="12" t="str">
-        <x:v>Legacy CardPG term</x:v>
-      </x:c>
-      <x:c r="C5" s="12" t="str">
-        <x:v>Dealbreak term</x:v>
-      </x:c>
-      <x:c r="D5" s="12" t="str">
-        <x:v>Area</x:v>
-      </x:c>
-      <x:c r="E5" s="12" t="str">
-        <x:v>Migration guidance</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="40" customHeight="1">
-      <x:c r="A6" s="3" t="str">
-        <x:v>Project title</x:v>
-      </x:c>
-      <x:c r="B6" s="3" t="str">
-        <x:v>CardPG</x:v>
-      </x:c>
-      <x:c r="C6" s="3" t="str">
-        <x:v>Dealbreak</x:v>
-      </x:c>
-      <x:c r="D6" s="3" t="str">
-        <x:v>Brand</x:v>
-      </x:c>
-      <x:c r="E6" s="3" t="str">
-        <x:v>Working title; verify trademark/store availability before release.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="25" customHeight="1">
-      <x:c r="A7" s="3" t="str">
-        <x:v>Currency</x:v>
-      </x:c>
-      <x:c r="B7" s="3" t="str">
-        <x:v>Gold</x:v>
-      </x:c>
-      <x:c r="C7" s="3" t="str">
-        <x:v>Credits</x:v>
-      </x:c>
-      <x:c r="D7" s="3" t="str">
-        <x:v>Economy</x:v>
-      </x:c>
-      <x:c r="E7" s="3" t="str">
-        <x:v>Amounts remain identical.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="40" customHeight="1">
-      <x:c r="A8" s="3" t="str">
-        <x:v>Equipment category</x:v>
-      </x:c>
-      <x:c r="B8" s="3" t="str">
-        <x:v>Artifact</x:v>
-      </x:c>
-      <x:c r="C8" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="D8" s="3" t="str">
-        <x:v>Inventory</x:v>
-      </x:c>
-      <x:c r="E8" s="3" t="str">
-        <x:v>Workbook IDs gear_*; original Unity rel_* IDs remain in Rename Index.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="40" customHeight="1">
-      <x:c r="A9" s="3" t="str">
-        <x:v>Card upgrades</x:v>
-      </x:c>
-      <x:c r="B9" s="3" t="str">
-        <x:v>Enhancement</x:v>
-      </x:c>
-      <x:c r="C9" s="3" t="str">
-        <x:v>Mod</x:v>
-      </x:c>
-      <x:c r="D9" s="3" t="str">
-        <x:v>Card systems</x:v>
-      </x:c>
-      <x:c r="E9" s="3" t="str">
-        <x:v>Workbook IDs mod_*; original Unity enh_* IDs remain in Rename Index.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="40" customHeight="1">
-      <x:c r="A10" s="3" t="str">
-        <x:v>One-use items</x:v>
-      </x:c>
-      <x:c r="B10" s="3" t="str">
-        <x:v>Consumable</x:v>
-      </x:c>
-      <x:c r="C10" s="3" t="str">
-        <x:v>Trick</x:v>
-      </x:c>
-      <x:c r="D10" s="3" t="str">
-        <x:v>Inventory</x:v>
-      </x:c>
-      <x:c r="E10" s="3" t="str">
-        <x:v>Workbook IDs consumable_*; Legacy Unity con_* IDs are retained in Rename Index.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="25" customHeight="1">
-      <x:c r="A11" s="3" t="str">
-        <x:v>Commerce</x:v>
-      </x:c>
-      <x:c r="B11" s="3" t="str">
-        <x:v>Shop</x:v>
-      </x:c>
-      <x:c r="C11" s="3" t="str">
-        <x:v>Black Market</x:v>
-      </x:c>
-      <x:c r="D11" s="3" t="str">
-        <x:v>Map / UI</x:v>
-      </x:c>
-      <x:c r="E11" s="3" t="str">
-        <x:v>Same shop mechanics and service offerings.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="25" customHeight="1">
-      <x:c r="A12" s="3" t="str">
-        <x:v>Special route encounter</x:v>
-      </x:c>
-      <x:c r="B12" s="3" t="str">
-        <x:v>Event</x:v>
-      </x:c>
-      <x:c r="C12" s="3" t="str">
-        <x:v>Incident</x:v>
-      </x:c>
-      <x:c r="D12" s="3" t="str">
-        <x:v>Map</x:v>
-      </x:c>
-      <x:c r="E12" s="3" t="str">
-        <x:v>Risk node mechanics unchanged.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="25" customHeight="1">
-      <x:c r="A13" s="3" t="str">
-        <x:v>Run segment</x:v>
-      </x:c>
-      <x:c r="B13" s="3" t="str">
-        <x:v>Map</x:v>
-      </x:c>
-      <x:c r="C13" s="3" t="str">
-        <x:v>District</x:v>
-      </x:c>
-      <x:c r="D13" s="3" t="str">
-        <x:v>Progression</x:v>
-      </x:c>
-      <x:c r="E13" s="3" t="str">
-        <x:v>12 districts; existing route depths unchanged.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="25" customHeight="1">
-      <x:c r="A14" s="3" t="str">
-        <x:v>Enforcer enemy</x:v>
-      </x:c>
-      <x:c r="B14" s="3" t="str">
-        <x:v>Elite</x:v>
-      </x:c>
-      <x:c r="C14" s="3" t="str">
-        <x:v>Enforcer</x:v>
-      </x:c>
-      <x:c r="D14" s="3" t="str">
-        <x:v>Combat</x:v>
-      </x:c>
-      <x:c r="E14" s="3" t="str">
-        <x:v>Enforcer flags and rewards unchanged.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="25" customHeight="1">
-      <x:c r="A15" s="3" t="str">
-        <x:v>Headliner enemy</x:v>
-      </x:c>
-      <x:c r="B15" s="3" t="str">
-        <x:v>Boss</x:v>
-      </x:c>
-      <x:c r="C15" s="3" t="str">
-        <x:v>Headliner</x:v>
-      </x:c>
-      <x:c r="D15" s="3" t="str">
-        <x:v>Combat</x:v>
-      </x:c>
-      <x:c r="E15" s="3" t="str">
-        <x:v>Headliner fight rank/suit and rewards unchanged.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="25" customHeight="1">
-      <x:c r="A16" s="3" t="str">
-        <x:v>Jacks tier</x:v>
-      </x:c>
-      <x:c r="B16" s="3" t="str">
-        <x:v>Jack</x:v>
-      </x:c>
-      <x:c r="C16" s="3" t="str">
-        <x:v>J / Runner tier</x:v>
-      </x:c>
-      <x:c r="D16" s="3" t="str">
-        <x:v>12 boss lineup</x:v>
-      </x:c>
-      <x:c r="E16" s="3" t="str">
-        <x:v>Display alias only; rank 11 is still Jack.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="25" customHeight="1">
-      <x:c r="A17" s="3" t="str">
-        <x:v>Queens tier</x:v>
-      </x:c>
-      <x:c r="B17" s="3" t="str">
-        <x:v>Queen</x:v>
-      </x:c>
-      <x:c r="C17" s="3" t="str">
-        <x:v>Q / Operator tier</x:v>
-      </x:c>
-      <x:c r="D17" s="3" t="str">
-        <x:v>12 boss lineup</x:v>
-      </x:c>
-      <x:c r="E17" s="3" t="str">
-        <x:v>Display alias only; rank 12 is still Queen.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="25" customHeight="1">
-      <x:c r="A18" s="3" t="str">
-        <x:v>Kings tier</x:v>
-      </x:c>
-      <x:c r="B18" s="3" t="str">
-        <x:v>King</x:v>
-      </x:c>
-      <x:c r="C18" s="3" t="str">
-        <x:v>K / Kingpin tier</x:v>
-      </x:c>
-      <x:c r="D18" s="3" t="str">
-        <x:v>12 boss lineup</x:v>
-      </x:c>
-      <x:c r="E18" s="3" t="str">
-        <x:v>Display alias only; rank 13 is still King.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="25" customHeight="1">
-      <x:c r="A19" s="3" t="str">
-        <x:v>Map navigation</x:v>
-      </x:c>
-      <x:c r="B19" s="3" t="str">
-        <x:v>Node</x:v>
-      </x:c>
-      <x:c r="C19" s="3" t="str">
-        <x:v>Node</x:v>
-      </x:c>
-      <x:c r="D19" s="3" t="str">
-        <x:v>UI / topology</x:v>
-      </x:c>
-      <x:c r="E19" s="3" t="str">
-        <x:v>Keep technical route-node terminology.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="25" customHeight="1">
-      <x:c r="A20" s="3" t="str">
-        <x:v>Defense</x:v>
-      </x:c>
-      <x:c r="B20" s="3" t="str">
-        <x:v>Block</x:v>
-      </x:c>
-      <x:c r="C20" s="3" t="str">
-        <x:v>Block</x:v>
-      </x:c>
-      <x:c r="D20" s="3" t="str">
-        <x:v>Combat</x:v>
-      </x:c>
-      <x:c r="E20" s="3" t="str">
-        <x:v>Do not rename or alter Perfect Block.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="25" customHeight="1">
-      <x:c r="A21" s="3" t="str">
-        <x:v>Damage absorption</x:v>
-      </x:c>
-      <x:c r="B21" s="3" t="str">
-        <x:v>Shield</x:v>
-      </x:c>
-      <x:c r="C21" s="3" t="str">
-        <x:v>Shield</x:v>
-      </x:c>
-      <x:c r="D21" s="3" t="str">
-        <x:v>Combat</x:v>
-      </x:c>
-      <x:c r="E21" s="3" t="str">
-        <x:v>Distinct from Block; mechanics unchanged.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="40" customHeight="1">
-      <x:c r="A22" s="3" t="str">
-        <x:v>Card identities</x:v>
-      </x:c>
-      <x:c r="B22" s="3" t="str">
-        <x:v>Hearts / Diamonds / Clubs / Spades</x:v>
-      </x:c>
-      <x:c r="C22" s="3" t="str">
-        <x:v>Hearts / Diamonds / Clubs / Spades</x:v>
-      </x:c>
-      <x:c r="D22" s="3" t="str">
-        <x:v>Cards</x:v>
-      </x:c>
-      <x:c r="E22" s="3" t="str">
-        <x:v>Same physical suits and card ranks.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="25" customHeight="1">
-      <x:c r="A23" s="3" t="str">
-        <x:v>Headliner reward</x:v>
-      </x:c>
-      <x:c r="B23" s="3" t="str">
-        <x:v>Exact Face Card</x:v>
-      </x:c>
-      <x:c r="C23" s="3" t="str">
-        <x:v>Exact J/Q/K face card</x:v>
-      </x:c>
-      <x:c r="D23" s="3" t="str">
-        <x:v>Rewards</x:v>
-      </x:c>
-      <x:c r="E23" s="3" t="str">
-        <x:v>Exact rank + suit inserted into the deck.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" ht="25" customHeight="1">
-      <x:c r="A24" s="3" t="str">
-        <x:v>Shop service</x:v>
-      </x:c>
-      <x:c r="B24" s="3" t="str">
-        <x:v>Investment</x:v>
-      </x:c>
-      <x:c r="C24" s="3" t="str">
-        <x:v>Stake</x:v>
-      </x:c>
-      <x:c r="D24" s="3" t="str">
-        <x:v>Black Market</x:v>
-      </x:c>
-      <x:c r="E24" s="3" t="str">
-        <x:v>Same risk and payout.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" ht="25" customHeight="1">
-      <x:c r="A25" s="3" t="str">
-        <x:v>Shop service</x:v>
-      </x:c>
-      <x:c r="B25" s="3" t="str">
-        <x:v>Guidance</x:v>
-      </x:c>
-      <x:c r="C25" s="3" t="str">
-        <x:v>Intel</x:v>
-      </x:c>
-      <x:c r="D25" s="3" t="str">
-        <x:v>Black Market</x:v>
-      </x:c>
-      <x:c r="E25" s="3" t="str">
-        <x:v>Same node reveal.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26" ht="25" customHeight="1">
-      <x:c r="A26" s="3" t="str">
-        <x:v>Shop service</x:v>
-      </x:c>
-      <x:c r="B26" s="3" t="str">
-        <x:v>Quest</x:v>
-      </x:c>
-      <x:c r="C26" s="3" t="str">
-        <x:v>Contract</x:v>
-      </x:c>
-      <x:c r="D26" s="3" t="str">
-        <x:v>Black Market</x:v>
-      </x:c>
-      <x:c r="E26" s="3" t="str">
-        <x:v>Same objectives and penalties.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="25" customHeight="1">
-      <x:c r="A27" s="3" t="str">
-        <x:v>Poker finisher</x:v>
-      </x:c>
-      <x:c r="B27" s="3" t="str">
-        <x:v>Royal Straight Flush</x:v>
-      </x:c>
-      <x:c r="C27" s="3" t="str">
-        <x:v>Royal Flush</x:v>
-      </x:c>
-      <x:c r="D27" s="3" t="str">
-        <x:v>Finisher</x:v>
-      </x:c>
-      <x:c r="E27" s="3" t="str">
-        <x:v>Still specifically 10/J/Q/K/A of one effective suit.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28" ht="25" customHeight="1">
-      <x:c r="A28" s="3"/>
-      <x:c r="B28" s="3"/>
-      <x:c r="C28" s="3"/>
-      <x:c r="D28" s="3"/>
-      <x:c r="E28" s="3"/>
-    </x:row>
-    <x:row r="29" ht="25" customHeight="1">
-      <x:c r="A29" s="3"/>
-      <x:c r="B29" s="3"/>
-      <x:c r="C29" s="3"/>
-      <x:c r="D29" s="3"/>
-      <x:c r="E29" s="3"/>
-    </x:row>
-    <x:row r="30" ht="28" customHeight="1">
-      <x:c r="A30" s="22" t="str">
-        <x:v>INTEGRATION &amp; BOUNDARIES</x:v>
-      </x:c>
-      <x:c r="B30" s="22"/>
-      <x:c r="C30" s="22"/>
-      <x:c r="D30" s="22"/>
-      <x:c r="E30" s="22"/>
-    </x:row>
-    <x:row r="31" ht="130" customHeight="1">
-      <x:c r="A31" s="3" t="str">
-        <x:v>IDs remain stable</x:v>
-      </x:c>
-      <x:c r="B31" s="3" t="str">
-        <x:v>Canonical workbook IDs are retained during cleanup: foe_*, headliner_*, gear_*, mod_*, consumable_*, incident_*, service_*, node_* and headliner_ability_*. Legacy Unity IDs remain in Rename Index.</x:v>
-      </x:c>
-      <x:c r="C31" s="3"/>
-      <x:c r="D31" s="3"/>
-      <x:c r="E31" s="3"/>
-    </x:row>
-    <x:row r="32" ht="70" customHeight="1">
-      <x:c r="A32" s="3" t="str">
-        <x:v>Spreadsheet tabs kept</x:v>
-      </x:c>
-      <x:c r="B32" s="3" t="str">
-        <x:v>Legacy worksheet tab names are retained for compatibility with import scripts and existing references.</x:v>
-      </x:c>
-      <x:c r="C32" s="3"/>
-      <x:c r="D32" s="3"/>
-      <x:c r="E32" s="3"/>
-    </x:row>
-    <x:row r="33" ht="115" customHeight="1">
-      <x:c r="A33" s="3" t="str">
-        <x:v>Schema caution</x:v>
-      </x:c>
-      <x:c r="B33" s="3" t="str">
-        <x:v>Player-facing terms use Credits, Gear, Mod, Trick, District, Enforcer, Headliner, Black Market and Incident. Name-based importers need the corresponding terminology mapping.</x:v>
-      </x:c>
-      <x:c r="C33" s="3"/>
-      <x:c r="D33" s="3"/>
-      <x:c r="E33" s="3"/>
-    </x:row>
-    <x:row r="34" ht="85" customHeight="1">
-      <x:c r="A34" s="3" t="str">
-        <x:v>Runtime unchanged</x:v>
-      </x:c>
-      <x:c r="B34" s="3" t="str">
-        <x:v>Changing this workbook does not rename Unity assets, class types, scripts, UI labels, localization keys or saved data.</x:v>
-      </x:c>
-      <x:c r="C34" s="3"/>
-      <x:c r="D34" s="3"/>
-      <x:c r="E34" s="3"/>
-    </x:row>
-    <x:row r="35" ht="70" customHeight="1">
-      <x:c r="A35" s="3" t="str">
-        <x:v>Status unchanged</x:v>
-      </x:c>
-      <x:c r="B35" s="3" t="str">
-        <x:v>Implemented/Draft statuses are inherited. Workbook renames are not proof of Unity migration.</x:v>
-      </x:c>
-      <x:c r="C35" s="3"/>
-      <x:c r="D35" s="3"/>
-      <x:c r="E35" s="3"/>
-    </x:row>
-    <x:row r="36" ht="70" customHeight="1">
-      <x:c r="A36" s="3" t="str">
-        <x:v>No rebalance</x:v>
-      </x:c>
-      <x:c r="B36" s="3" t="str">
-        <x:v>All HP, ATK, prices, odds, drops, effects, tiers, reward sizes, sources and upgrade links are retained.</x:v>
-      </x:c>
-      <x:c r="C36" s="3"/>
-      <x:c r="D36" s="3"/>
-      <x:c r="E36" s="3"/>
-    </x:row>
-    <x:row r="37" ht="85" customHeight="1">
-      <x:c r="A37" s="3" t="str">
-        <x:v>Portrait direction</x:v>
-      </x:c>
-      <x:c r="B37" s="3" t="str">
-        <x:v>Graphic 2D portraits; modern street/corporate surrealism, punchy silhouettes, restrained color, suited J/Q/K aliases.</x:v>
-      </x:c>
-      <x:c r="C37" s="3"/>
-      <x:c r="D37" s="3"/>
-      <x:c r="E37" s="3"/>
-    </x:row>
-    <x:row r="38" ht="85" customHeight="1">
-      <x:c r="A38" s="3" t="str">
-        <x:v>Special encounter</x:v>
-      </x:c>
-      <x:c r="B38" s="3" t="str">
-        <x:v>headliner_013 / The House remains an undefined optional placeholder, not a new designed combat encounter.</x:v>
-      </x:c>
-      <x:c r="C38" s="3"/>
-      <x:c r="D38" s="3"/>
-      <x:c r="E38" s="3"/>
-    </x:row>
-    <x:row r="39" ht="85" customHeight="1">
-      <x:c r="A39" s="3" t="str">
-        <x:v>Source note</x:v>
-      </x:c>
-      <x:c r="B39" s="3" t="str">
-        <x:v>IDs and terminology were standardized in this workbook; Unity references and save data require separate migration.</x:v>
-      </x:c>
-      <x:c r="C39" s="3"/>
-      <x:c r="D39" s="3"/>
-      <x:c r="E39" s="3"/>
-    </x:row>
-  </x:sheetData>
-  <x:mergeCells>
-    <x:mergeCell ref="A1:E1"/>
-    <x:mergeCell ref="A2:E2"/>
-    <x:mergeCell ref="A4:E4"/>
-    <x:mergeCell ref="A30:E30"/>
-  </x:mergeCells>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="34" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="32" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="32" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="36" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="58" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="32" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="31" customHeight="1">
-      <x:c r="A1" s="19" t="str">
-        <x:v>DEALBREAK  /  CANONICAL NAME CROSSWALK</x:v>
-      </x:c>
-      <x:c r="B1" s="3"/>
-      <x:c r="C1" s="3"/>
-      <x:c r="D1" s="3"/>
-      <x:c r="E1" s="3"/>
-      <x:c r="F1" s="3"/>
-      <x:c r="G1" s="3"/>
-    </x:row>
-    <x:row r="2" ht="35" customHeight="1">
-      <x:c r="A2" s="20" t="str">
-        <x:v>Dealbreak IDs are canonical; see Legacy Unity ID for asset/code migration.</x:v>
-      </x:c>
-      <x:c r="B2" s="3"/>
-      <x:c r="C2" s="3"/>
-      <x:c r="D2" s="3"/>
-      <x:c r="E2" s="3"/>
-      <x:c r="F2" s="3"/>
-      <x:c r="G2" s="3"/>
-    </x:row>
-    <x:row r="3" ht="24" customHeight="1">
-      <x:c r="A3" s="3"/>
-      <x:c r="B3" s="3"/>
-      <x:c r="C3" s="3"/>
-      <x:c r="D3" s="3"/>
-      <x:c r="E3" s="3"/>
-      <x:c r="F3" s="3"/>
-      <x:c r="G3" s="3"/>
-    </x:row>
-    <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="12" t="str">
-        <x:v>Sheet (legacy)</x:v>
-      </x:c>
-      <x:c r="B4" s="12" t="str">
-        <x:v>Dealbreak ID</x:v>
-      </x:c>
-      <x:c r="C4" s="12" t="str">
-        <x:v>Original name</x:v>
-      </x:c>
-      <x:c r="D4" s="12" t="str">
-        <x:v>Dealbreak display name</x:v>
-      </x:c>
-      <x:c r="E4" s="12" t="str">
-        <x:v>Status</x:v>
-      </x:c>
-      <x:c r="F4" s="12" t="str">
-        <x:v>Migration note</x:v>
-      </x:c>
-      <x:c r="G4" s="12" t="str">
-        <x:v>Legacy Unity ID</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="25" customHeight="1">
-      <x:c r="A5" s="3" t="str">
-        <x:v>Enemies</x:v>
-      </x:c>
-      <x:c r="B5" s="3" t="str">
-        <x:v>foe_goblin</x:v>
-      </x:c>
-      <x:c r="C5" s="3" t="str">
-        <x:v>Goblin</x:v>
-      </x:c>
-      <x:c r="D5" s="3" t="str">
-        <x:v>Scrapper</x:v>
-      </x:c>
-      <x:c r="E5" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F5" s="3" t="str">
-        <x:v>Same HP/ATK, AI design and drop</x:v>
-      </x:c>
-      <x:c r="G5" s="3" t="str">
-        <x:v>enemy_goblin</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="25" customHeight="1">
-      <x:c r="A6" s="3" t="str">
-        <x:v>Enemies</x:v>
-      </x:c>
-      <x:c r="B6" s="3" t="str">
-        <x:v>foe_thief</x:v>
-      </x:c>
-      <x:c r="C6" s="3" t="str">
-        <x:v>Thief</x:v>
-      </x:c>
-      <x:c r="D6" s="3" t="str">
-        <x:v>Pickpocket</x:v>
-      </x:c>
-      <x:c r="E6" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F6" s="3" t="str">
-        <x:v>Same HP/ATK, AI design and drop</x:v>
-      </x:c>
-      <x:c r="G6" s="3" t="str">
-        <x:v>enemy_thief</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="25" customHeight="1">
-      <x:c r="A7" s="3" t="str">
-        <x:v>Enemies</x:v>
-      </x:c>
-      <x:c r="B7" s="3" t="str">
-        <x:v>foe_knight</x:v>
-      </x:c>
-      <x:c r="C7" s="3" t="str">
-        <x:v>Knight</x:v>
-      </x:c>
-      <x:c r="D7" s="3" t="str">
-        <x:v>Security Guard</x:v>
-      </x:c>
-      <x:c r="E7" s="3" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="F7" s="3" t="str">
-        <x:v>Same HP/ATK, AI design and drop</x:v>
-      </x:c>
-      <x:c r="G7" s="3" t="str">
-        <x:v>enemy_knight</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="25" customHeight="1">
-      <x:c r="A8" s="3" t="str">
-        <x:v>Enemies</x:v>
-      </x:c>
-      <x:c r="B8" s="3" t="str">
-        <x:v>foe_brute</x:v>
-      </x:c>
-      <x:c r="C8" s="3" t="str">
-        <x:v>Brute</x:v>
-      </x:c>
-      <x:c r="D8" s="3" t="str">
-        <x:v>Heavy</x:v>
-      </x:c>
-      <x:c r="E8" s="3" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="F8" s="3" t="str">
-        <x:v>Same HP/ATK, AI design and drop</x:v>
-      </x:c>
-      <x:c r="G8" s="3" t="str">
-        <x:v>enemy_brute</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="25" customHeight="1">
-      <x:c r="A9" s="3" t="str">
-        <x:v>Enemies</x:v>
-      </x:c>
-      <x:c r="B9" s="3" t="str">
-        <x:v>foe_shieldbearer</x:v>
-      </x:c>
-      <x:c r="C9" s="3" t="str">
-        <x:v>Shieldbearer</x:v>
-      </x:c>
-      <x:c r="D9" s="3" t="str">
-        <x:v>Riot Guard</x:v>
-      </x:c>
-      <x:c r="E9" s="3" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="F9" s="3" t="str">
-        <x:v>Same HP/ATK, AI design and drop</x:v>
-      </x:c>
-      <x:c r="G9" s="3" t="str">
-        <x:v>enemy_shieldbearer</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="25" customHeight="1">
-      <x:c r="A10" s="3" t="str">
-        <x:v>Enemies</x:v>
-      </x:c>
-      <x:c r="B10" s="3" t="str">
-        <x:v>foe_war_drummer</x:v>
-      </x:c>
-      <x:c r="C10" s="3" t="str">
-        <x:v>War Drummer</x:v>
-      </x:c>
-      <x:c r="D10" s="3" t="str">
-        <x:v>Hype Man</x:v>
-      </x:c>
-      <x:c r="E10" s="3" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="F10" s="3" t="str">
-        <x:v>Same HP/ATK, AI design and drop</x:v>
-      </x:c>
-      <x:c r="G10" s="3" t="str">
-        <x:v>enemy_war_drummer</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="25" customHeight="1">
-      <x:c r="A11" s="3" t="str">
-        <x:v>Enemies</x:v>
-      </x:c>
-      <x:c r="B11" s="3" t="str">
-        <x:v>foe_duelist</x:v>
-      </x:c>
-      <x:c r="C11" s="3" t="str">
-        <x:v>Duelist</x:v>
-      </x:c>
-      <x:c r="D11" s="3" t="str">
-        <x:v>Challenger</x:v>
-      </x:c>
-      <x:c r="E11" s="3" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="F11" s="3" t="str">
-        <x:v>Same HP/ATK, AI design and drop</x:v>
-      </x:c>
-      <x:c r="G11" s="3" t="str">
-        <x:v>enemy_duelist</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="25" customHeight="1">
-      <x:c r="A12" s="3" t="str">
-        <x:v>Enemies</x:v>
-      </x:c>
-      <x:c r="B12" s="3" t="str">
-        <x:v>foe_goblin_captain</x:v>
-      </x:c>
-      <x:c r="C12" s="3" t="str">
-        <x:v>Goblin Captain</x:v>
-      </x:c>
-      <x:c r="D12" s="3" t="str">
-        <x:v>Crew Leader</x:v>
-      </x:c>
-      <x:c r="E12" s="3" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="F12" s="3" t="str">
-        <x:v>Same HP/ATK, AI design and drop</x:v>
-      </x:c>
-      <x:c r="G12" s="3" t="str">
-        <x:v>enemy_goblin_captain</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="25" customHeight="1">
-      <x:c r="A13" s="3" t="str">
-        <x:v>Enemies</x:v>
-      </x:c>
-      <x:c r="B13" s="3" t="str">
-        <x:v>foe_royal_knight</x:v>
-      </x:c>
-      <x:c r="C13" s="3" t="str">
-        <x:v>Royal Knight</x:v>
-      </x:c>
-      <x:c r="D13" s="3" t="str">
-        <x:v>Riot Captain</x:v>
-      </x:c>
-      <x:c r="E13" s="3" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="F13" s="3" t="str">
-        <x:v>Same HP/ATK, AI design and drop</x:v>
-      </x:c>
-      <x:c r="G13" s="3" t="str">
-        <x:v>enemy_royal_knight</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="40" customHeight="1">
-      <x:c r="A14" s="3" t="str">
-        <x:v>Enemies</x:v>
-      </x:c>
-      <x:c r="B14" s="3" t="str">
-        <x:v>foe_master_thief</x:v>
-      </x:c>
-      <x:c r="C14" s="3" t="str">
-        <x:v>Master Thief</x:v>
-      </x:c>
-      <x:c r="D14" s="3" t="str">
-        <x:v>Ghost</x:v>
-      </x:c>
-      <x:c r="E14" s="3" t="str">
-        <x:v>Implemented — awaiting phase acceptance</x:v>
-      </x:c>
-      <x:c r="F14" s="3" t="str">
-        <x:v>Same HP/ATK, AI design and drop</x:v>
-      </x:c>
-      <x:c r="G14" s="3" t="str">
-        <x:v>enemy_master_thief</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="25" customHeight="1">
-      <x:c r="A15" s="3" t="str">
-        <x:v>Headliners</x:v>
-      </x:c>
-      <x:c r="B15" s="3" t="str">
-        <x:v>headliner_001</x:v>
-      </x:c>
-      <x:c r="C15" s="3" t="str">
-        <x:v>Jack of Hearts</x:v>
-      </x:c>
-      <x:c r="D15" s="3" t="str">
-        <x:v>J♥ — The Charmer</x:v>
-      </x:c>
-      <x:c r="E15" s="3" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="F15" s="3" t="str">
-        <x:v>Rank/suit/face-card reward unchanged</x:v>
-      </x:c>
-      <x:c r="G15" s="3" t="str">
-        <x:v>boss_001</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="25" customHeight="1">
-      <x:c r="A16" s="3" t="str">
-        <x:v>Headliners</x:v>
-      </x:c>
-      <x:c r="B16" s="3" t="str">
-        <x:v>headliner_002</x:v>
-      </x:c>
-      <x:c r="C16" s="3" t="str">
-        <x:v>Jack of Diamonds</x:v>
-      </x:c>
-      <x:c r="D16" s="3" t="str">
-        <x:v>J♦ — The Courier</x:v>
-      </x:c>
-      <x:c r="E16" s="3" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="F16" s="3" t="str">
-        <x:v>Rank/suit/face-card reward unchanged</x:v>
-      </x:c>
-      <x:c r="G16" s="3" t="str">
-        <x:v>boss_002</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="25" customHeight="1">
-      <x:c r="A17" s="3" t="str">
-        <x:v>Headliners</x:v>
-      </x:c>
-      <x:c r="B17" s="3" t="str">
-        <x:v>headliner_003</x:v>
-      </x:c>
-      <x:c r="C17" s="3" t="str">
-        <x:v>Jack of Clubs</x:v>
-      </x:c>
-      <x:c r="D17" s="3" t="str">
-        <x:v>J♣ — The Hitter</x:v>
-      </x:c>
-      <x:c r="E17" s="3" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="F17" s="3" t="str">
-        <x:v>Rank/suit/face-card reward unchanged</x:v>
-      </x:c>
-      <x:c r="G17" s="3" t="str">
-        <x:v>boss_003</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="25" customHeight="1">
-      <x:c r="A18" s="3" t="str">
-        <x:v>Headliners</x:v>
-      </x:c>
-      <x:c r="B18" s="3" t="str">
-        <x:v>headliner_004</x:v>
-      </x:c>
-      <x:c r="C18" s="3" t="str">
-        <x:v>Jack of Spades</x:v>
-      </x:c>
-      <x:c r="D18" s="3" t="str">
-        <x:v>J♠ — The Fixer</x:v>
-      </x:c>
-      <x:c r="E18" s="3" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="F18" s="3" t="str">
-        <x:v>Rank/suit/face-card reward unchanged</x:v>
-      </x:c>
-      <x:c r="G18" s="3" t="str">
-        <x:v>boss_004</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="25" customHeight="1">
-      <x:c r="A19" s="3" t="str">
-        <x:v>Headliners</x:v>
-      </x:c>
-      <x:c r="B19" s="3" t="str">
-        <x:v>headliner_005</x:v>
-      </x:c>
-      <x:c r="C19" s="3" t="str">
-        <x:v>Queen of Hearts</x:v>
-      </x:c>
-      <x:c r="D19" s="3" t="str">
-        <x:v>Q♥ — The Influencer</x:v>
-      </x:c>
-      <x:c r="E19" s="3" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="F19" s="3" t="str">
-        <x:v>Rank/suit/face-card reward unchanged</x:v>
-      </x:c>
-      <x:c r="G19" s="3" t="str">
-        <x:v>boss_005</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="25" customHeight="1">
-      <x:c r="A20" s="3" t="str">
-        <x:v>Headliners</x:v>
-      </x:c>
-      <x:c r="B20" s="3" t="str">
-        <x:v>headliner_006</x:v>
-      </x:c>
-      <x:c r="C20" s="3" t="str">
-        <x:v>Queen of Diamonds</x:v>
-      </x:c>
-      <x:c r="D20" s="3" t="str">
-        <x:v>Q♦ — The Broker</x:v>
-      </x:c>
-      <x:c r="E20" s="3" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="F20" s="3" t="str">
-        <x:v>Rank/suit/face-card reward unchanged</x:v>
-      </x:c>
-      <x:c r="G20" s="3" t="str">
-        <x:v>boss_006</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="25" customHeight="1">
-      <x:c r="A21" s="3" t="str">
-        <x:v>Headliners</x:v>
-      </x:c>
-      <x:c r="B21" s="3" t="str">
-        <x:v>headliner_007</x:v>
-      </x:c>
-      <x:c r="C21" s="3" t="str">
-        <x:v>Queen of Clubs</x:v>
-      </x:c>
-      <x:c r="D21" s="3" t="str">
-        <x:v>Q♣ — The Foreman</x:v>
-      </x:c>
-      <x:c r="E21" s="3" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="F21" s="3" t="str">
-        <x:v>Rank/suit/face-card reward unchanged</x:v>
-      </x:c>
-      <x:c r="G21" s="3" t="str">
-        <x:v>boss_007</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="25" customHeight="1">
-      <x:c r="A22" s="3" t="str">
-        <x:v>Headliners</x:v>
-      </x:c>
-      <x:c r="B22" s="3" t="str">
-        <x:v>headliner_008</x:v>
-      </x:c>
-      <x:c r="C22" s="3" t="str">
-        <x:v>Queen of Spades</x:v>
-      </x:c>
-      <x:c r="D22" s="3" t="str">
-        <x:v>Q♠ — The Handler</x:v>
-      </x:c>
-      <x:c r="E22" s="3" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="F22" s="3" t="str">
-        <x:v>Rank/suit/face-card reward unchanged</x:v>
-      </x:c>
-      <x:c r="G22" s="3" t="str">
-        <x:v>boss_008</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="25" customHeight="1">
-      <x:c r="A23" s="3" t="str">
-        <x:v>Headliners</x:v>
-      </x:c>
-      <x:c r="B23" s="3" t="str">
-        <x:v>headliner_009</x:v>
-      </x:c>
-      <x:c r="C23" s="3" t="str">
-        <x:v>King of Hearts</x:v>
-      </x:c>
-      <x:c r="D23" s="3" t="str">
-        <x:v>K♥ — The Icon</x:v>
-      </x:c>
-      <x:c r="E23" s="3" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="F23" s="3" t="str">
-        <x:v>Rank/suit/face-card reward unchanged</x:v>
-      </x:c>
-      <x:c r="G23" s="3" t="str">
-        <x:v>boss_009</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" ht="25" customHeight="1">
-      <x:c r="A24" s="3" t="str">
-        <x:v>Headliners</x:v>
-      </x:c>
-      <x:c r="B24" s="3" t="str">
-        <x:v>headliner_010</x:v>
-      </x:c>
-      <x:c r="C24" s="3" t="str">
-        <x:v>King of Diamonds</x:v>
-      </x:c>
-      <x:c r="D24" s="3" t="str">
-        <x:v>K♦ — The Mogul</x:v>
-      </x:c>
-      <x:c r="E24" s="3" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="F24" s="3" t="str">
-        <x:v>Rank/suit/face-card reward unchanged</x:v>
-      </x:c>
-      <x:c r="G24" s="3" t="str">
-        <x:v>boss_010</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" ht="25" customHeight="1">
-      <x:c r="A25" s="3" t="str">
-        <x:v>Headliners</x:v>
-      </x:c>
-      <x:c r="B25" s="3" t="str">
-        <x:v>headliner_011</x:v>
-      </x:c>
-      <x:c r="C25" s="3" t="str">
-        <x:v>King of Clubs</x:v>
-      </x:c>
-      <x:c r="D25" s="3" t="str">
-        <x:v>K♣ — The Chairman</x:v>
-      </x:c>
-      <x:c r="E25" s="3" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="F25" s="3" t="str">
-        <x:v>Rank/suit/face-card reward unchanged</x:v>
-      </x:c>
-      <x:c r="G25" s="3" t="str">
-        <x:v>boss_011</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26" ht="25" customHeight="1">
-      <x:c r="A26" s="3" t="str">
-        <x:v>Headliners</x:v>
-      </x:c>
-      <x:c r="B26" s="3" t="str">
-        <x:v>headliner_012</x:v>
-      </x:c>
-      <x:c r="C26" s="3" t="str">
-        <x:v>King of Spades</x:v>
-      </x:c>
-      <x:c r="D26" s="3" t="str">
-        <x:v>K♠ — The Director</x:v>
-      </x:c>
-      <x:c r="E26" s="3" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="F26" s="3" t="str">
-        <x:v>Rank/suit/face-card reward unchanged</x:v>
-      </x:c>
-      <x:c r="G26" s="3" t="str">
-        <x:v>boss_012</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="25" customHeight="1">
-      <x:c r="A27" s="3" t="str">
-        <x:v>Headliners</x:v>
-      </x:c>
-      <x:c r="B27" s="3" t="str">
-        <x:v>headliner_013</x:v>
-      </x:c>
-      <x:c r="C27" s="3" t="str">
-        <x:v>God</x:v>
-      </x:c>
-      <x:c r="D27" s="3" t="str">
-        <x:v>The House</x:v>
-      </x:c>
-      <x:c r="E27" s="3"/>
-      <x:c r="F27" s="3" t="str">
-        <x:v>Rank/suit/face-card reward unchanged</x:v>
-      </x:c>
-      <x:c r="G27" s="3" t="str">
-        <x:v>boss_013</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28" ht="25" customHeight="1">
-      <x:c r="A28" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B28" s="3" t="str">
-        <x:v>gear_101</x:v>
-      </x:c>
-      <x:c r="C28" s="3" t="str">
-        <x:v>Artisan Tools</x:v>
-      </x:c>
-      <x:c r="D28" s="3" t="str">
-        <x:v>Modder's Kit</x:v>
-      </x:c>
-      <x:c r="E28" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F28" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G28" s="3" t="str">
-        <x:v>rel_101</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29" ht="25" customHeight="1">
-      <x:c r="A29" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B29" s="3" t="str">
-        <x:v>gear_102</x:v>
-      </x:c>
-      <x:c r="C29" s="3" t="str">
-        <x:v>Golden Compass</x:v>
-      </x:c>
-      <x:c r="D29" s="3" t="str">
-        <x:v>Payout Tracker</x:v>
-      </x:c>
-      <x:c r="E29" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F29" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G29" s="3" t="str">
-        <x:v>rel_102</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30" ht="25" customHeight="1">
-      <x:c r="A30" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B30" s="3" t="str">
-        <x:v>gear_103</x:v>
-      </x:c>
-      <x:c r="C30" s="3" t="str">
-        <x:v>Reinforced Sleeves</x:v>
-      </x:c>
-      <x:c r="D30" s="3" t="str">
-        <x:v>Carbon Sleeves</x:v>
-      </x:c>
-      <x:c r="E30" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F30" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G30" s="3" t="str">
-        <x:v>rel_103</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" ht="25" customHeight="1">
-      <x:c r="A31" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B31" s="3" t="str">
-        <x:v>gear_104</x:v>
-      </x:c>
-      <x:c r="C31" s="3" t="str">
-        <x:v>Victory Draught</x:v>
-      </x:c>
-      <x:c r="D31" s="3" t="str">
-        <x:v>Recovery Can</x:v>
-      </x:c>
-      <x:c r="E31" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F31" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G31" s="3" t="str">
-        <x:v>rel_104</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32" ht="25" customHeight="1">
-      <x:c r="A32" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B32" s="3" t="str">
-        <x:v>gear_006</x:v>
-      </x:c>
-      <x:c r="C32" s="3" t="str">
-        <x:v>Dagger</x:v>
-      </x:c>
-      <x:c r="D32" s="3" t="str">
-        <x:v>Box Cutter</x:v>
-      </x:c>
-      <x:c r="E32" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F32" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G32" s="3" t="str">
-        <x:v>rel_006</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33" ht="25" customHeight="1">
-      <x:c r="A33" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B33" s="3" t="str">
-        <x:v>gear_019</x:v>
-      </x:c>
-      <x:c r="C33" s="3" t="str">
-        <x:v>Chain Armor</x:v>
-      </x:c>
-      <x:c r="D33" s="3" t="str">
-        <x:v>Tactical Plating</x:v>
-      </x:c>
-      <x:c r="E33" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F33" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G33" s="3" t="str">
-        <x:v>rel_019</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34" ht="25" customHeight="1">
-      <x:c r="A34" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B34" s="3" t="str">
-        <x:v>gear_005</x:v>
-      </x:c>
-      <x:c r="C34" s="3" t="str">
-        <x:v>Leather Armor</x:v>
-      </x:c>
-      <x:c r="D34" s="3" t="str">
-        <x:v>Street Jacket</x:v>
-      </x:c>
-      <x:c r="E34" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F34" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G34" s="3" t="str">
-        <x:v>rel_005</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35" ht="25" customHeight="1">
-      <x:c r="A35" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B35" s="3" t="str">
-        <x:v>gear_016</x:v>
-      </x:c>
-      <x:c r="C35" s="3" t="str">
-        <x:v>Retaliation Emblem</x:v>
-      </x:c>
-      <x:c r="D35" s="3" t="str">
-        <x:v>Payback Chip</x:v>
-      </x:c>
-      <x:c r="E35" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F35" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G35" s="3" t="str">
-        <x:v>rel_016</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="36" ht="25" customHeight="1">
-      <x:c r="A36" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B36" s="3" t="str">
-        <x:v>gear_022</x:v>
-      </x:c>
-      <x:c r="C36" s="3" t="str">
-        <x:v>Retaliation Emblem</x:v>
-      </x:c>
-      <x:c r="D36" s="3" t="str">
-        <x:v>Payback Chip</x:v>
-      </x:c>
-      <x:c r="E36" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F36" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G36" s="3" t="str">
-        <x:v>rel_022</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="37" ht="40" customHeight="1">
-      <x:c r="A37" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B37" s="3" t="str">
-        <x:v>gear_111</x:v>
-      </x:c>
-      <x:c r="C37" s="3" t="str">
-        <x:v>Retaliation Emblem</x:v>
-      </x:c>
-      <x:c r="D37" s="3" t="str">
-        <x:v>Payback Chip</x:v>
-      </x:c>
-      <x:c r="E37" s="3" t="str">
-        <x:v>Implemented — awaiting phase acceptance</x:v>
-      </x:c>
-      <x:c r="F37" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G37" s="3" t="str">
-        <x:v>rel_111</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="38" ht="40" customHeight="1">
-      <x:c r="A38" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B38" s="3" t="str">
-        <x:v>gear_139</x:v>
-      </x:c>
-      <x:c r="C38" s="3" t="str">
-        <x:v>Crown of Endurance</x:v>
-      </x:c>
-      <x:c r="D38" s="3" t="str">
-        <x:v>Survivor's Badge</x:v>
-      </x:c>
-      <x:c r="E38" s="3" t="str">
-        <x:v>Implemented — awaiting phase acceptance</x:v>
-      </x:c>
-      <x:c r="F38" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G38" s="3" t="str">
-        <x:v>rel_139</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="39" ht="40" customHeight="1">
-      <x:c r="A39" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B39" s="3" t="str">
-        <x:v>gear_138</x:v>
-      </x:c>
-      <x:c r="C39" s="3" t="str">
-        <x:v>Kingslayer's Mark</x:v>
-      </x:c>
-      <x:c r="D39" s="3" t="str">
-        <x:v>Headliner Tag</x:v>
-      </x:c>
-      <x:c r="E39" s="3" t="str">
-        <x:v>Implemented — awaiting phase acceptance</x:v>
-      </x:c>
-      <x:c r="F39" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G39" s="3" t="str">
-        <x:v>rel_138</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="40" ht="25" customHeight="1">
-      <x:c r="A40" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B40" s="3" t="str">
-        <x:v>gear_001</x:v>
-      </x:c>
-      <x:c r="C40" s="3" t="str">
-        <x:v>Club Emblem</x:v>
-      </x:c>
-      <x:c r="D40" s="3" t="str">
-        <x:v>Club Amplifier</x:v>
-      </x:c>
-      <x:c r="E40" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F40" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G40" s="3" t="str">
-        <x:v>rel_001</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="41" ht="25" customHeight="1">
-      <x:c r="A41" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B41" s="3" t="str">
-        <x:v>gear_025</x:v>
-      </x:c>
-      <x:c r="C41" s="3" t="str">
-        <x:v>Club Emblem</x:v>
-      </x:c>
-      <x:c r="D41" s="3" t="str">
-        <x:v>Club Amplifier</x:v>
-      </x:c>
-      <x:c r="E41" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F41" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G41" s="3" t="str">
-        <x:v>rel_025</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="42" ht="40" customHeight="1">
-      <x:c r="A42" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B42" s="3" t="str">
-        <x:v>gear_034</x:v>
-      </x:c>
-      <x:c r="C42" s="3" t="str">
-        <x:v>Club Emblem</x:v>
-      </x:c>
-      <x:c r="D42" s="3" t="str">
-        <x:v>Club Amplifier</x:v>
-      </x:c>
-      <x:c r="E42" s="3" t="str">
-        <x:v>Implemented — awaiting phase acceptance</x:v>
-      </x:c>
-      <x:c r="F42" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G42" s="3" t="str">
-        <x:v>rel_034</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="43" ht="40" customHeight="1">
-      <x:c r="A43" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B43" s="3" t="str">
-        <x:v>gear_123</x:v>
-      </x:c>
-      <x:c r="C43" s="3" t="str">
-        <x:v>Preparation Manual</x:v>
-      </x:c>
-      <x:c r="D43" s="3" t="str">
-        <x:v>Preflight Checklist</x:v>
-      </x:c>
-      <x:c r="E43" s="3" t="str">
-        <x:v>Implemented — awaiting phase acceptance</x:v>
-      </x:c>
-      <x:c r="F43" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G43" s="3" t="str">
-        <x:v>rel_123</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="44" ht="40" customHeight="1">
-      <x:c r="A44" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B44" s="3" t="str">
-        <x:v>gear_117</x:v>
-      </x:c>
-      <x:c r="C44" s="3" t="str">
-        <x:v>Scavenger's Pouch</x:v>
-      </x:c>
-      <x:c r="D44" s="3" t="str">
-        <x:v>Salvage Pouch</x:v>
-      </x:c>
-      <x:c r="E44" s="3" t="str">
-        <x:v>Implemented — awaiting phase acceptance</x:v>
-      </x:c>
-      <x:c r="F44" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G44" s="3" t="str">
-        <x:v>rel_117</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="45" ht="40" customHeight="1">
-      <x:c r="A45" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B45" s="3" t="str">
-        <x:v>gear_129</x:v>
-      </x:c>
-      <x:c r="C45" s="3" t="str">
-        <x:v>Scavenger's Satchel</x:v>
-      </x:c>
-      <x:c r="D45" s="3" t="str">
-        <x:v>Salvage Bag</x:v>
-      </x:c>
-      <x:c r="E45" s="3" t="str">
-        <x:v>Implemented — awaiting phase acceptance</x:v>
-      </x:c>
-      <x:c r="F45" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G45" s="3" t="str">
-        <x:v>rel_129</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="46" ht="40" customHeight="1">
-      <x:c r="A46" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B46" s="3" t="str">
-        <x:v>gear_120</x:v>
-      </x:c>
-      <x:c r="C46" s="3" t="str">
-        <x:v>Traveler's Pack</x:v>
-      </x:c>
-      <x:c r="D46" s="3" t="str">
-        <x:v>Carry Rig</x:v>
-      </x:c>
-      <x:c r="E46" s="3" t="str">
-        <x:v>Implemented — awaiting phase acceptance</x:v>
-      </x:c>
-      <x:c r="F46" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G46" s="3" t="str">
-        <x:v>rel_120</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="47" ht="40" customHeight="1">
-      <x:c r="A47" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B47" s="3" t="str">
-        <x:v>gear_121</x:v>
-      </x:c>
-      <x:c r="C47" s="3" t="str">
-        <x:v>Traveler's Pack</x:v>
-      </x:c>
-      <x:c r="D47" s="3" t="str">
-        <x:v>Carry Rig</x:v>
-      </x:c>
-      <x:c r="E47" s="3" t="str">
-        <x:v>Implemented — awaiting phase acceptance</x:v>
-      </x:c>
-      <x:c r="F47" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G47" s="3" t="str">
-        <x:v>rel_121</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="48" ht="25" customHeight="1">
-      <x:c r="A48" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B48" s="3" t="str">
-        <x:v>gear_014</x:v>
-      </x:c>
-      <x:c r="C48" s="3" t="str">
-        <x:v>Ace Emblem</x:v>
-      </x:c>
-      <x:c r="D48" s="3" t="str">
-        <x:v>Ace Protocol</x:v>
-      </x:c>
-      <x:c r="E48" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F48" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G48" s="3" t="str">
-        <x:v>rel_014</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="49" ht="40" customHeight="1">
-      <x:c r="A49" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B49" s="3" t="str">
-        <x:v>gear_114</x:v>
-      </x:c>
-      <x:c r="C49" s="3" t="str">
-        <x:v>Ace Emblem</x:v>
-      </x:c>
-      <x:c r="D49" s="3" t="str">
-        <x:v>Ace Protocol</x:v>
-      </x:c>
-      <x:c r="E49" s="3" t="str">
-        <x:v>Implemented — awaiting phase acceptance</x:v>
-      </x:c>
-      <x:c r="F49" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G49" s="3" t="str">
-        <x:v>rel_114</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="50" ht="40" customHeight="1">
-      <x:c r="A50" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B50" s="3" t="str">
-        <x:v>gear_115</x:v>
-      </x:c>
-      <x:c r="C50" s="3" t="str">
-        <x:v>Ace Emblem</x:v>
-      </x:c>
-      <x:c r="D50" s="3" t="str">
-        <x:v>Ace Protocol</x:v>
-      </x:c>
-      <x:c r="E50" s="3" t="str">
-        <x:v>Implemented — awaiting phase acceptance</x:v>
-      </x:c>
-      <x:c r="F50" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G50" s="3" t="str">
-        <x:v>rel_115</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="51" ht="25" customHeight="1">
-      <x:c r="A51" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B51" s="3" t="str">
-        <x:v>gear_023</x:v>
-      </x:c>
-      <x:c r="C51" s="3" t="str">
-        <x:v>Sword</x:v>
-      </x:c>
-      <x:c r="D51" s="3" t="str">
-        <x:v>Power Baton</x:v>
-      </x:c>
-      <x:c r="E51" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F51" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G51" s="3" t="str">
-        <x:v>rel_023</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="52" ht="25" customHeight="1">
-      <x:c r="A52" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B52" s="3" t="str">
-        <x:v>gear_018</x:v>
-      </x:c>
-      <x:c r="C52" s="3" t="str">
-        <x:v>Fire Emblem</x:v>
-      </x:c>
-      <x:c r="D52" s="3" t="str">
-        <x:v>Burn Notice</x:v>
-      </x:c>
-      <x:c r="E52" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F52" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G52" s="3" t="str">
-        <x:v>rel_018</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="53" ht="25" customHeight="1">
-      <x:c r="A53" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B53" s="3" t="str">
-        <x:v>gear_003</x:v>
-      </x:c>
-      <x:c r="C53" s="3" t="str">
-        <x:v>Diamond Emblem</x:v>
-      </x:c>
-      <x:c r="D53" s="3" t="str">
-        <x:v>Diamond Driver</x:v>
-      </x:c>
-      <x:c r="E53" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F53" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G53" s="3" t="str">
-        <x:v>rel_003</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="54" ht="25" customHeight="1">
-      <x:c r="A54" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B54" s="3" t="str">
-        <x:v>gear_027</x:v>
-      </x:c>
-      <x:c r="C54" s="3" t="str">
-        <x:v>Diamond Emblem</x:v>
-      </x:c>
-      <x:c r="D54" s="3" t="str">
-        <x:v>Diamond Driver</x:v>
-      </x:c>
-      <x:c r="E54" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F54" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G54" s="3" t="str">
-        <x:v>rel_027</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="55" ht="40" customHeight="1">
-      <x:c r="A55" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B55" s="3" t="str">
-        <x:v>gear_108</x:v>
-      </x:c>
-      <x:c r="C55" s="3" t="str">
-        <x:v>Diamond Emblem</x:v>
-      </x:c>
-      <x:c r="D55" s="3" t="str">
-        <x:v>Diamond Driver</x:v>
-      </x:c>
-      <x:c r="E55" s="3" t="str">
-        <x:v>Implemented — awaiting phase acceptance</x:v>
-      </x:c>
-      <x:c r="F55" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G55" s="3" t="str">
-        <x:v>rel_108</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="56" ht="25" customHeight="1">
-      <x:c r="A56" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B56" s="3" t="str">
-        <x:v>gear_015</x:v>
-      </x:c>
-      <x:c r="C56" s="3" t="str">
-        <x:v>Overflow Emblem</x:v>
-      </x:c>
-      <x:c r="D56" s="3" t="str">
-        <x:v>Overflow Script</x:v>
-      </x:c>
-      <x:c r="E56" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F56" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G56" s="3" t="str">
-        <x:v>rel_015</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="57" ht="25" customHeight="1">
-      <x:c r="A57" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B57" s="3" t="str">
-        <x:v>gear_021</x:v>
-      </x:c>
-      <x:c r="C57" s="3" t="str">
-        <x:v>Overflow Emblem</x:v>
-      </x:c>
-      <x:c r="D57" s="3" t="str">
-        <x:v>Overflow Script</x:v>
-      </x:c>
-      <x:c r="E57" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F57" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G57" s="3" t="str">
-        <x:v>rel_021</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="58" ht="40" customHeight="1">
-      <x:c r="A58" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B58" s="3" t="str">
-        <x:v>gear_110</x:v>
-      </x:c>
-      <x:c r="C58" s="3" t="str">
-        <x:v>Overflow Emblem</x:v>
-      </x:c>
-      <x:c r="D58" s="3" t="str">
-        <x:v>Overflow Script</x:v>
-      </x:c>
-      <x:c r="E58" s="3" t="str">
-        <x:v>Implemented — awaiting phase acceptance</x:v>
-      </x:c>
-      <x:c r="F58" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G58" s="3" t="str">
-        <x:v>rel_110</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="59" ht="25" customHeight="1">
-      <x:c r="A59" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B59" s="3" t="str">
-        <x:v>gear_007</x:v>
-      </x:c>
-      <x:c r="C59" s="3" t="str">
-        <x:v>Tome</x:v>
-      </x:c>
-      <x:c r="D59" s="3" t="str">
-        <x:v>Pocket Guide</x:v>
-      </x:c>
-      <x:c r="E59" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F59" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G59" s="3" t="str">
-        <x:v>rel_007</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="60" ht="40" customHeight="1">
-      <x:c r="A60" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B60" s="3" t="str">
-        <x:v>gear_126</x:v>
-      </x:c>
-      <x:c r="C60" s="3" t="str">
-        <x:v>Bounty Ledger</x:v>
-      </x:c>
-      <x:c r="D60" s="3" t="str">
-        <x:v>Hit List</x:v>
-      </x:c>
-      <x:c r="E60" s="3" t="str">
-        <x:v>Implemented — awaiting phase acceptance</x:v>
-      </x:c>
-      <x:c r="F60" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G60" s="3" t="str">
-        <x:v>rel_126</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="61" ht="40" customHeight="1">
-      <x:c r="A61" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B61" s="3" t="str">
-        <x:v>gear_125</x:v>
-      </x:c>
-      <x:c r="C61" s="3" t="str">
-        <x:v>Cashback Token</x:v>
-      </x:c>
-      <x:c r="D61" s="3" t="str">
-        <x:v>Cashback Card</x:v>
-      </x:c>
-      <x:c r="E61" s="3" t="str">
-        <x:v>Implemented — awaiting phase acceptance</x:v>
-      </x:c>
-      <x:c r="F61" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G61" s="3" t="str">
-        <x:v>rel_125</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="62" ht="40" customHeight="1">
-      <x:c r="A62" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B62" s="3" t="str">
-        <x:v>gear_128</x:v>
-      </x:c>
-      <x:c r="C62" s="3" t="str">
-        <x:v>Gilded Blade</x:v>
-      </x:c>
-      <x:c r="D62" s="3" t="str">
-        <x:v>Cash Cutter</x:v>
-      </x:c>
-      <x:c r="E62" s="3" t="str">
-        <x:v>Implemented — awaiting phase acceptance</x:v>
-      </x:c>
-      <x:c r="F62" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G62" s="3" t="str">
-        <x:v>rel_128</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="63" ht="40" customHeight="1">
-      <x:c r="A63" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B63" s="3" t="str">
-        <x:v>gear_127</x:v>
-      </x:c>
-      <x:c r="C63" s="3" t="str">
-        <x:v>Golden Vault</x:v>
-      </x:c>
-      <x:c r="D63" s="3" t="str">
-        <x:v>Savings Account</x:v>
-      </x:c>
-      <x:c r="E63" s="3" t="str">
-        <x:v>Implemented — awaiting phase acceptance</x:v>
-      </x:c>
-      <x:c r="F63" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G63" s="3" t="str">
-        <x:v>rel_127</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="64" ht="40" customHeight="1">
-      <x:c r="A64" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B64" s="3" t="str">
-        <x:v>gear_124</x:v>
-      </x:c>
-      <x:c r="C64" s="3" t="str">
-        <x:v>Merchant's Badge</x:v>
-      </x:c>
-      <x:c r="D64" s="3" t="str">
-        <x:v>Loyalty Card</x:v>
-      </x:c>
-      <x:c r="E64" s="3" t="str">
-        <x:v>Implemented — awaiting phase acceptance</x:v>
-      </x:c>
-      <x:c r="F64" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G64" s="3" t="str">
-        <x:v>rel_124</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="65" ht="40" customHeight="1">
-      <x:c r="A65" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B65" s="3" t="str">
-        <x:v>gear_131</x:v>
-      </x:c>
-      <x:c r="C65" s="3" t="str">
-        <x:v>Merchant's Gift</x:v>
-      </x:c>
-      <x:c r="D65" s="3" t="str">
-        <x:v>Loyalty Perk</x:v>
-      </x:c>
-      <x:c r="E65" s="3" t="str">
-        <x:v>Implemented — awaiting phase acceptance</x:v>
-      </x:c>
-      <x:c r="F65" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G65" s="3" t="str">
-        <x:v>rel_131</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="66" ht="40" customHeight="1">
-      <x:c r="A66" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B66" s="3" t="str">
-        <x:v>gear_136</x:v>
-      </x:c>
-      <x:c r="C66" s="3" t="str">
-        <x:v>Challenger's Crest</x:v>
-      </x:c>
-      <x:c r="D66" s="3" t="str">
-        <x:v>Challenger Patch</x:v>
-      </x:c>
-      <x:c r="E66" s="3" t="str">
-        <x:v>Implemented — awaiting phase acceptance</x:v>
-      </x:c>
-      <x:c r="F66" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G66" s="3" t="str">
-        <x:v>rel_136</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="67" ht="40" customHeight="1">
-      <x:c r="A67" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B67" s="3" t="str">
-        <x:v>gear_137</x:v>
-      </x:c>
-      <x:c r="C67" s="3" t="str">
-        <x:v>Trophy Rack</x:v>
-      </x:c>
-      <x:c r="D67" s="3" t="str">
-        <x:v>Victory Wall</x:v>
-      </x:c>
-      <x:c r="E67" s="3" t="str">
-        <x:v>Implemented — awaiting phase acceptance</x:v>
-      </x:c>
-      <x:c r="F67" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G67" s="3" t="str">
-        <x:v>rel_137</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="68" ht="40" customHeight="1">
-      <x:c r="A68" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B68" s="3" t="str">
-        <x:v>gear_119</x:v>
-      </x:c>
-      <x:c r="C68" s="3" t="str">
-        <x:v>Hunter's Ledger</x:v>
-      </x:c>
-      <x:c r="D68" s="3" t="str">
-        <x:v>Takedown Log</x:v>
-      </x:c>
-      <x:c r="E68" s="3" t="str">
-        <x:v>Implemented — awaiting phase acceptance</x:v>
-      </x:c>
-      <x:c r="F68" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G68" s="3" t="str">
-        <x:v>rel_119</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="69" ht="40" customHeight="1">
-      <x:c r="A69" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B69" s="3" t="str">
-        <x:v>gear_130</x:v>
-      </x:c>
-      <x:c r="C69" s="3" t="str">
-        <x:v>Alchemist's Kit</x:v>
-      </x:c>
-      <x:c r="D69" s="3" t="str">
-        <x:v>Mod Supply Kit</x:v>
-      </x:c>
-      <x:c r="E69" s="3" t="str">
-        <x:v>Implemented — awaiting phase acceptance</x:v>
-      </x:c>
-      <x:c r="F69" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G69" s="3" t="str">
-        <x:v>rel_130</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="70" ht="25" customHeight="1">
-      <x:c r="A70" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B70" s="3" t="str">
-        <x:v>gear_009</x:v>
-      </x:c>
-      <x:c r="C70" s="3" t="str">
-        <x:v>Hammer</x:v>
-      </x:c>
-      <x:c r="D70" s="3" t="str">
-        <x:v>Mod Bench</x:v>
-      </x:c>
-      <x:c r="E70" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F70" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G70" s="3" t="str">
-        <x:v>rel_009</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="71" ht="40" customHeight="1">
-      <x:c r="A71" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B71" s="3" t="str">
-        <x:v>gear_140</x:v>
-      </x:c>
-      <x:c r="C71" s="3" t="str">
-        <x:v>Hammer</x:v>
-      </x:c>
-      <x:c r="D71" s="3" t="str">
-        <x:v>Mod Bench</x:v>
-      </x:c>
-      <x:c r="E71" s="3" t="str">
-        <x:v>Implemented — awaiting phase acceptance</x:v>
-      </x:c>
-      <x:c r="F71" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G71" s="3" t="str">
-        <x:v>rel_140</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="72" ht="25" customHeight="1">
-      <x:c r="A72" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B72" s="3" t="str">
-        <x:v>gear_031</x:v>
-      </x:c>
-      <x:c r="C72" s="3" t="str">
-        <x:v>Glass Emblem</x:v>
-      </x:c>
-      <x:c r="D72" s="3" t="str">
-        <x:v>Glass Mode</x:v>
-      </x:c>
-      <x:c r="E72" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F72" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G72" s="3" t="str">
-        <x:v>rel_031</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="73" ht="25" customHeight="1">
-      <x:c r="A73" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B73" s="3" t="str">
-        <x:v>gear_032</x:v>
-      </x:c>
-      <x:c r="C73" s="3" t="str">
-        <x:v>Glass Emblem</x:v>
-      </x:c>
-      <x:c r="D73" s="3" t="str">
-        <x:v>Glass Mode</x:v>
-      </x:c>
-      <x:c r="E73" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F73" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G73" s="3" t="str">
-        <x:v>rel_032</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="74" ht="25" customHeight="1">
-      <x:c r="A74" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B74" s="3" t="str">
-        <x:v>gear_033</x:v>
-      </x:c>
-      <x:c r="C74" s="3" t="str">
-        <x:v>Glass Emblem</x:v>
-      </x:c>
-      <x:c r="D74" s="3" t="str">
-        <x:v>Glass Mode</x:v>
-      </x:c>
-      <x:c r="E74" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F74" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G74" s="3" t="str">
-        <x:v>rel_033</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="75" ht="25" customHeight="1">
-      <x:c r="A75" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B75" s="3" t="str">
-        <x:v>gear_028</x:v>
-      </x:c>
-      <x:c r="C75" s="3" t="str">
-        <x:v>Arsenal Emblem</x:v>
-      </x:c>
-      <x:c r="D75" s="3" t="str">
-        <x:v>Extra Slots</x:v>
-      </x:c>
-      <x:c r="E75" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F75" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G75" s="3" t="str">
-        <x:v>rel_028</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="76" ht="25" customHeight="1">
-      <x:c r="A76" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B76" s="3" t="str">
-        <x:v>gear_029</x:v>
-      </x:c>
-      <x:c r="C76" s="3" t="str">
-        <x:v>Arsenal Emblem</x:v>
-      </x:c>
-      <x:c r="D76" s="3" t="str">
-        <x:v>Extra Slots</x:v>
-      </x:c>
-      <x:c r="E76" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F76" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G76" s="3" t="str">
-        <x:v>rel_029</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="77" ht="40" customHeight="1">
-      <x:c r="A77" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B77" s="3" t="str">
-        <x:v>gear_030</x:v>
-      </x:c>
-      <x:c r="C77" s="3" t="str">
-        <x:v>Arsenal Emblem</x:v>
-      </x:c>
-      <x:c r="D77" s="3" t="str">
-        <x:v>Extra Slots</x:v>
-      </x:c>
-      <x:c r="E77" s="3" t="str">
-        <x:v>Implemented — awaiting phase acceptance</x:v>
-      </x:c>
-      <x:c r="F77" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G77" s="3" t="str">
-        <x:v>rel_030</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="78" ht="40" customHeight="1">
-      <x:c r="A78" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B78" s="3" t="str">
-        <x:v>gear_122</x:v>
-      </x:c>
-      <x:c r="C78" s="3" t="str">
-        <x:v>Field Medic's Kit</x:v>
-      </x:c>
-      <x:c r="D78" s="3" t="str">
-        <x:v>First-Aid Kit</x:v>
-      </x:c>
-      <x:c r="E78" s="3" t="str">
-        <x:v>Implemented — awaiting phase acceptance</x:v>
-      </x:c>
-      <x:c r="F78" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G78" s="3" t="str">
-        <x:v>rel_122</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="79" ht="25" customHeight="1">
-      <x:c r="A79" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B79" s="3" t="str">
-        <x:v>gear_010</x:v>
-      </x:c>
-      <x:c r="C79" s="3" t="str">
-        <x:v>Healing Light</x:v>
-      </x:c>
-      <x:c r="D79" s="3" t="str">
-        <x:v>Auto-Injector</x:v>
-      </x:c>
-      <x:c r="E79" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F79" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G79" s="3" t="str">
-        <x:v>rel_010</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="80" ht="25" customHeight="1">
-      <x:c r="A80" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B80" s="3" t="str">
-        <x:v>gear_002</x:v>
-      </x:c>
-      <x:c r="C80" s="3" t="str">
-        <x:v>Heart Emblem</x:v>
-      </x:c>
-      <x:c r="D80" s="3" t="str">
-        <x:v>Heartbeat Chip</x:v>
-      </x:c>
-      <x:c r="E80" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F80" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G80" s="3" t="str">
-        <x:v>rel_002</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="81" ht="25" customHeight="1">
-      <x:c r="A81" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B81" s="3" t="str">
-        <x:v>gear_026</x:v>
-      </x:c>
-      <x:c r="C81" s="3" t="str">
-        <x:v>Heart Emblem</x:v>
-      </x:c>
-      <x:c r="D81" s="3" t="str">
-        <x:v>Heartbeat Chip</x:v>
-      </x:c>
-      <x:c r="E81" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F81" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G81" s="3" t="str">
-        <x:v>rel_026</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="82" ht="40" customHeight="1">
-      <x:c r="A82" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B82" s="3" t="str">
-        <x:v>gear_105</x:v>
-      </x:c>
-      <x:c r="C82" s="3" t="str">
-        <x:v>Heart Emblem</x:v>
-      </x:c>
-      <x:c r="D82" s="3" t="str">
-        <x:v>Heartbeat Chip</x:v>
-      </x:c>
-      <x:c r="E82" s="3" t="str">
-        <x:v>Implemented — awaiting phase acceptance</x:v>
-      </x:c>
-      <x:c r="F82" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G82" s="3" t="str">
-        <x:v>rel_105</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="83" ht="25" customHeight="1">
-      <x:c r="A83" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B83" s="3" t="str">
-        <x:v>gear_017</x:v>
-      </x:c>
-      <x:c r="C83" s="3" t="str">
-        <x:v>Mimic Emblem</x:v>
-      </x:c>
-      <x:c r="D83" s="3" t="str">
-        <x:v>Echo Driver</x:v>
-      </x:c>
-      <x:c r="E83" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F83" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G83" s="3" t="str">
-        <x:v>rel_017</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="84" ht="40" customHeight="1">
-      <x:c r="A84" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B84" s="3" t="str">
-        <x:v>gear_116</x:v>
-      </x:c>
-      <x:c r="C84" s="3" t="str">
-        <x:v>Mimic Emblem</x:v>
-      </x:c>
-      <x:c r="D84" s="3" t="str">
-        <x:v>Echo Driver</x:v>
-      </x:c>
-      <x:c r="E84" s="3" t="str">
-        <x:v>Implemented — awaiting phase acceptance</x:v>
-      </x:c>
-      <x:c r="F84" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G84" s="3" t="str">
-        <x:v>rel_116</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="85" ht="25" customHeight="1">
-      <x:c r="A85" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B85" s="3" t="str">
-        <x:v>gear_013</x:v>
-      </x:c>
-      <x:c r="C85" s="3" t="str">
-        <x:v>Dwarf Emblem</x:v>
-      </x:c>
-      <x:c r="D85" s="3" t="str">
-        <x:v>Lowball Protocol</x:v>
-      </x:c>
-      <x:c r="E85" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F85" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G85" s="3" t="str">
-        <x:v>rel_013</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="86" ht="40" customHeight="1">
-      <x:c r="A86" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B86" s="3" t="str">
-        <x:v>gear_112</x:v>
-      </x:c>
-      <x:c r="C86" s="3" t="str">
-        <x:v>Dwarf Emblem</x:v>
-      </x:c>
-      <x:c r="D86" s="3" t="str">
-        <x:v>Lowball Protocol</x:v>
-      </x:c>
-      <x:c r="E86" s="3" t="str">
-        <x:v>Implemented — awaiting phase acceptance</x:v>
-      </x:c>
-      <x:c r="F86" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G86" s="3" t="str">
-        <x:v>rel_112</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="87" ht="40" customHeight="1">
-      <x:c r="A87" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B87" s="3" t="str">
-        <x:v>gear_113</x:v>
-      </x:c>
-      <x:c r="C87" s="3" t="str">
-        <x:v>Dwarf Emblem</x:v>
-      </x:c>
-      <x:c r="D87" s="3" t="str">
-        <x:v>Lowball Protocol</x:v>
-      </x:c>
-      <x:c r="E87" s="3" t="str">
-        <x:v>Implemented — awaiting phase acceptance</x:v>
-      </x:c>
-      <x:c r="F87" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G87" s="3" t="str">
-        <x:v>rel_113</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="88" ht="40" customHeight="1">
-      <x:c r="A88" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B88" s="3" t="str">
-        <x:v>gear_135</x:v>
-      </x:c>
-      <x:c r="C88" s="3" t="str">
-        <x:v>Hidden Trail</x:v>
-      </x:c>
-      <x:c r="D88" s="3" t="str">
-        <x:v>Side Door</x:v>
-      </x:c>
-      <x:c r="E88" s="3" t="str">
-        <x:v>Implemented — awaiting phase acceptance</x:v>
-      </x:c>
-      <x:c r="F88" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G88" s="3" t="str">
-        <x:v>rel_135</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="89" ht="25" customHeight="1">
-      <x:c r="A89" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B89" s="3" t="str">
-        <x:v>gear_008</x:v>
-      </x:c>
-      <x:c r="C89" s="3" t="str">
-        <x:v>Lantern</x:v>
-      </x:c>
-      <x:c r="D89" s="3" t="str">
-        <x:v>Scanner</x:v>
-      </x:c>
-      <x:c r="E89" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F89" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G89" s="3" t="str">
-        <x:v>rel_008</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="90" ht="40" customHeight="1">
-      <x:c r="A90" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B90" s="3" t="str">
-        <x:v>gear_132</x:v>
-      </x:c>
-      <x:c r="C90" s="3" t="str">
-        <x:v>Surveyor's Map</x:v>
-      </x:c>
-      <x:c r="D90" s="3" t="str">
-        <x:v>Network Map</x:v>
-      </x:c>
-      <x:c r="E90" s="3" t="str">
-        <x:v>Deferred by owner — redundant visibility; not implemented</x:v>
-      </x:c>
-      <x:c r="F90" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G90" s="3" t="str">
-        <x:v>rel_132</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="91" ht="40" customHeight="1">
-      <x:c r="A91" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B91" s="3" t="str">
-        <x:v>gear_133</x:v>
-      </x:c>
-      <x:c r="C91" s="3" t="str">
-        <x:v>Wanderer's Boots</x:v>
-      </x:c>
-      <x:c r="D91" s="3" t="str">
-        <x:v>City Sneakers</x:v>
-      </x:c>
-      <x:c r="E91" s="3" t="str">
-        <x:v>Implemented — awaiting phase acceptance</x:v>
-      </x:c>
-      <x:c r="F91" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G91" s="3" t="str">
-        <x:v>rel_133</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="92" ht="40" customHeight="1">
-      <x:c r="A92" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B92" s="3" t="str">
-        <x:v>gear_134</x:v>
-      </x:c>
-      <x:c r="C92" s="3" t="str">
-        <x:v>Warpath Banner</x:v>
-      </x:c>
-      <x:c r="D92" s="3" t="str">
-        <x:v>Win-Streak Patch</x:v>
-      </x:c>
-      <x:c r="E92" s="3" t="str">
-        <x:v>Implemented — awaiting phase acceptance</x:v>
-      </x:c>
-      <x:c r="F92" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G92" s="3" t="str">
-        <x:v>rel_134</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="93" ht="25" customHeight="1">
-      <x:c r="A93" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B93" s="3" t="str">
-        <x:v>gear_012</x:v>
-      </x:c>
-      <x:c r="C93" s="3" t="str">
-        <x:v>Hands Emblem</x:v>
-      </x:c>
-      <x:c r="D93" s="3" t="str">
-        <x:v>Combo Driver</x:v>
-      </x:c>
-      <x:c r="E93" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F93" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G93" s="3" t="str">
-        <x:v>rel_012</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="94" ht="25" customHeight="1">
-      <x:c r="A94" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B94" s="3" t="str">
-        <x:v>gear_020</x:v>
-      </x:c>
-      <x:c r="C94" s="3" t="str">
-        <x:v>Hands Emblem</x:v>
-      </x:c>
-      <x:c r="D94" s="3" t="str">
-        <x:v>Combo Driver</x:v>
-      </x:c>
-      <x:c r="E94" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F94" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G94" s="3" t="str">
-        <x:v>rel_020</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="95" ht="40" customHeight="1">
-      <x:c r="A95" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B95" s="3" t="str">
-        <x:v>gear_109</x:v>
-      </x:c>
-      <x:c r="C95" s="3" t="str">
-        <x:v>Hands Emblem</x:v>
-      </x:c>
-      <x:c r="D95" s="3" t="str">
-        <x:v>Combo Driver</x:v>
-      </x:c>
-      <x:c r="E95" s="3" t="str">
-        <x:v>Implemented — awaiting phase acceptance</x:v>
-      </x:c>
-      <x:c r="F95" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G95" s="3" t="str">
-        <x:v>rel_109</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="96" ht="25" customHeight="1">
-      <x:c r="A96" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B96" s="3" t="str">
-        <x:v>gear_100</x:v>
-      </x:c>
-      <x:c r="C96" s="3" t="str">
-        <x:v>Royal Family Heirloom</x:v>
-      </x:c>
-      <x:c r="D96" s="3" t="str">
-        <x:v>Royal Override</x:v>
-      </x:c>
-      <x:c r="E96" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F96" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G96" s="3" t="str">
-        <x:v>rel_100</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="97" ht="40" customHeight="1">
-      <x:c r="A97" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B97" s="3" t="str">
-        <x:v>gear_118</x:v>
-      </x:c>
-      <x:c r="C97" s="3" t="str">
-        <x:v>Balancer's Scale</x:v>
-      </x:c>
-      <x:c r="D97" s="3" t="str">
-        <x:v>Flip Switch</x:v>
-      </x:c>
-      <x:c r="E97" s="3" t="str">
-        <x:v>Implemented — awaiting phase acceptance</x:v>
-      </x:c>
-      <x:c r="F97" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G97" s="3" t="str">
-        <x:v>rel_118</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="98" ht="25" customHeight="1">
-      <x:c r="A98" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B98" s="3" t="str">
-        <x:v>gear_004</x:v>
-      </x:c>
-      <x:c r="C98" s="3" t="str">
-        <x:v>Spade Emblem</x:v>
-      </x:c>
-      <x:c r="D98" s="3" t="str">
-        <x:v>Spade Shield</x:v>
-      </x:c>
-      <x:c r="E98" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F98" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G98" s="3" t="str">
-        <x:v>rel_004</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="99" ht="40" customHeight="1">
-      <x:c r="A99" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B99" s="3" t="str">
-        <x:v>gear_106</x:v>
-      </x:c>
-      <x:c r="C99" s="3" t="str">
-        <x:v>Spade Emblem</x:v>
-      </x:c>
-      <x:c r="D99" s="3" t="str">
-        <x:v>Spade Shield</x:v>
-      </x:c>
-      <x:c r="E99" s="3" t="str">
-        <x:v>Implemented — awaiting phase acceptance</x:v>
-      </x:c>
-      <x:c r="F99" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G99" s="3" t="str">
-        <x:v>rel_106</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="100" ht="40" customHeight="1">
-      <x:c r="A100" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B100" s="3" t="str">
-        <x:v>gear_107</x:v>
-      </x:c>
-      <x:c r="C100" s="3" t="str">
-        <x:v>Spade Emblem</x:v>
-      </x:c>
-      <x:c r="D100" s="3" t="str">
-        <x:v>Spade Shield</x:v>
-      </x:c>
-      <x:c r="E100" s="3" t="str">
-        <x:v>Implemented — awaiting phase acceptance</x:v>
-      </x:c>
-      <x:c r="F100" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G100" s="3" t="str">
-        <x:v>rel_107</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="101" ht="25" customHeight="1">
-      <x:c r="A101" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B101" s="3" t="str">
-        <x:v>gear_011</x:v>
-      </x:c>
-      <x:c r="C101" s="3" t="str">
-        <x:v>Cheater Emblem</x:v>
-      </x:c>
-      <x:c r="D101" s="3" t="str">
-        <x:v>Extra Move</x:v>
-      </x:c>
-      <x:c r="E101" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F101" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G101" s="3" t="str">
-        <x:v>rel_011</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="102" ht="25" customHeight="1">
-      <x:c r="A102" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B102" s="3" t="str">
-        <x:v>gear_024</x:v>
-      </x:c>
-      <x:c r="C102" s="3" t="str">
-        <x:v>Cheater Emblem</x:v>
-      </x:c>
-      <x:c r="D102" s="3" t="str">
-        <x:v>Extra Move</x:v>
-      </x:c>
-      <x:c r="E102" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F102" s="3" t="str">
-        <x:v>Same tier/upgrade links and effect values</x:v>
-      </x:c>
-      <x:c r="G102" s="3" t="str">
-        <x:v>rel_024</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="103" ht="25" customHeight="1">
-      <x:c r="A103" s="3" t="str">
-        <x:v>Mods</x:v>
-      </x:c>
-      <x:c r="B103" s="3" t="str">
-        <x:v>mod_001</x:v>
-      </x:c>
-      <x:c r="C103" s="3" t="str">
-        <x:v>Sharpened</x:v>
-      </x:c>
-      <x:c r="D103" s="3" t="str">
-        <x:v>Boosted</x:v>
-      </x:c>
-      <x:c r="E103" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F103" s="3" t="str">
-        <x:v>Same card Mod trigger and effect</x:v>
-      </x:c>
-      <x:c r="G103" s="3" t="str">
-        <x:v>enh_001</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="104" ht="25" customHeight="1">
-      <x:c r="A104" s="3" t="str">
-        <x:v>Mods</x:v>
-      </x:c>
-      <x:c r="B104" s="3" t="str">
-        <x:v>mod_002</x:v>
-      </x:c>
-      <x:c r="C104" s="3" t="str">
-        <x:v>Hardened</x:v>
-      </x:c>
-      <x:c r="D104" s="3" t="str">
-        <x:v>Plated</x:v>
-      </x:c>
-      <x:c r="E104" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F104" s="3" t="str">
-        <x:v>Same card Mod trigger and effect</x:v>
-      </x:c>
-      <x:c r="G104" s="3" t="str">
-        <x:v>enh_002</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="105" ht="25" customHeight="1">
-      <x:c r="A105" s="3" t="str">
-        <x:v>Mods</x:v>
-      </x:c>
-      <x:c r="B105" s="3" t="str">
-        <x:v>mod_003</x:v>
-      </x:c>
-      <x:c r="C105" s="3" t="str">
-        <x:v>Mending</x:v>
-      </x:c>
-      <x:c r="D105" s="3" t="str">
-        <x:v>Regenerative</x:v>
-      </x:c>
-      <x:c r="E105" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F105" s="3" t="str">
-        <x:v>Same card Mod trigger and effect</x:v>
-      </x:c>
-      <x:c r="G105" s="3" t="str">
-        <x:v>enh_003</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="106" ht="25" customHeight="1">
-      <x:c r="A106" s="3" t="str">
-        <x:v>Mods</x:v>
-      </x:c>
-      <x:c r="B106" s="3" t="str">
-        <x:v>mod_004</x:v>
-      </x:c>
-      <x:c r="C106" s="3" t="str">
-        <x:v>Quickdraw</x:v>
-      </x:c>
-      <x:c r="D106" s="3" t="str">
-        <x:v>Quickload</x:v>
-      </x:c>
-      <x:c r="E106" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F106" s="3" t="str">
-        <x:v>Same card Mod trigger and effect</x:v>
-      </x:c>
-      <x:c r="G106" s="3" t="str">
-        <x:v>enh_004</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="107" ht="25" customHeight="1">
-      <x:c r="A107" s="3" t="str">
-        <x:v>Mods</x:v>
-      </x:c>
-      <x:c r="B107" s="3" t="str">
-        <x:v>mod_005</x:v>
-      </x:c>
-      <x:c r="C107" s="3" t="str">
-        <x:v>Devouring</x:v>
-      </x:c>
-      <x:c r="D107" s="3" t="str">
-        <x:v>Predatory</x:v>
-      </x:c>
-      <x:c r="E107" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F107" s="3" t="str">
-        <x:v>Same card Mod trigger and effect</x:v>
-      </x:c>
-      <x:c r="G107" s="3" t="str">
-        <x:v>enh_005</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="108" ht="25" customHeight="1">
-      <x:c r="A108" s="3" t="str">
-        <x:v>Mods</x:v>
-      </x:c>
-      <x:c r="B108" s="3" t="str">
-        <x:v>mod_006</x:v>
-      </x:c>
-      <x:c r="C108" s="3" t="str">
-        <x:v>Lethal</x:v>
-      </x:c>
-      <x:c r="D108" s="3" t="str">
-        <x:v>Deadeye</x:v>
-      </x:c>
-      <x:c r="E108" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F108" s="3" t="str">
-        <x:v>Same card Mod trigger and effect</x:v>
-      </x:c>
-      <x:c r="G108" s="3" t="str">
-        <x:v>enh_006</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="109" ht="25" customHeight="1">
-      <x:c r="A109" s="3" t="str">
-        <x:v>Mods</x:v>
-      </x:c>
-      <x:c r="B109" s="3" t="str">
-        <x:v>mod_007</x:v>
-      </x:c>
-      <x:c r="C109" s="3" t="str">
-        <x:v>Golden</x:v>
-      </x:c>
-      <x:c r="D109" s="3" t="str">
-        <x:v>Profitable</x:v>
-      </x:c>
-      <x:c r="E109" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F109" s="3" t="str">
-        <x:v>Same card Mod trigger and effect</x:v>
-      </x:c>
-      <x:c r="G109" s="3" t="str">
-        <x:v>enh_007</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="110" ht="25" customHeight="1">
-      <x:c r="A110" s="3" t="str">
-        <x:v>Mods</x:v>
-      </x:c>
-      <x:c r="B110" s="3" t="str">
-        <x:v>mod_008</x:v>
-      </x:c>
-      <x:c r="C110" s="3" t="str">
-        <x:v>Auxiliary</x:v>
-      </x:c>
-      <x:c r="D110" s="3" t="str">
-        <x:v>Backup</x:v>
-      </x:c>
-      <x:c r="E110" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F110" s="3" t="str">
-        <x:v>Same card Mod trigger and effect</x:v>
-      </x:c>
-      <x:c r="G110" s="3" t="str">
-        <x:v>enh_008</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="111" ht="25" customHeight="1">
-      <x:c r="A111" s="3" t="str">
-        <x:v>Mods</x:v>
-      </x:c>
-      <x:c r="B111" s="3" t="str">
-        <x:v>mod_009</x:v>
-      </x:c>
-      <x:c r="C111" s="3" t="str">
-        <x:v>Explosive</x:v>
-      </x:c>
-      <x:c r="D111" s="3" t="str">
-        <x:v>Volatile</x:v>
-      </x:c>
-      <x:c r="E111" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F111" s="3" t="str">
-        <x:v>Same card Mod trigger and effect</x:v>
-      </x:c>
-      <x:c r="G111" s="3" t="str">
-        <x:v>enh_009</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="112" ht="25" customHeight="1">
-      <x:c r="A112" s="3" t="str">
-        <x:v>Mods</x:v>
-      </x:c>
-      <x:c r="B112" s="3" t="str">
-        <x:v>mod_010</x:v>
-      </x:c>
-      <x:c r="C112" s="3" t="str">
-        <x:v>Vampiric</x:v>
-      </x:c>
-      <x:c r="D112" s="3" t="str">
-        <x:v>Overclocked</x:v>
-      </x:c>
-      <x:c r="E112" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F112" s="3" t="str">
-        <x:v>Same card Mod trigger and effect</x:v>
-      </x:c>
-      <x:c r="G112" s="3" t="str">
-        <x:v>enh_010</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="113" ht="25" customHeight="1">
-      <x:c r="A113" s="3" t="str">
-        <x:v>Mods</x:v>
-      </x:c>
-      <x:c r="B113" s="3" t="str">
-        <x:v>mod_011</x:v>
-      </x:c>
-      <x:c r="C113" s="3" t="str">
-        <x:v>Shifting</x:v>
-      </x:c>
-      <x:c r="D113" s="3" t="str">
-        <x:v>Wildcard</x:v>
-      </x:c>
-      <x:c r="E113" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F113" s="3" t="str">
-        <x:v>Same card Mod trigger and effect</x:v>
-      </x:c>
-      <x:c r="G113" s="3" t="str">
-        <x:v>enh_011</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="114" ht="25" customHeight="1">
-      <x:c r="A114" s="3" t="str">
-        <x:v>Events</x:v>
-      </x:c>
-      <x:c r="B114" s="3" t="str">
-        <x:v>incident_001</x:v>
-      </x:c>
-      <x:c r="C114" s="3" t="str">
-        <x:v>Roadside Cache</x:v>
-      </x:c>
-      <x:c r="D114" s="3" t="str">
-        <x:v>Dead Drop</x:v>
-      </x:c>
-      <x:c r="E114" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F114" s="3" t="str">
-        <x:v>Choice mechanics and outcomes unchanged</x:v>
-      </x:c>
-      <x:c r="G114" s="3" t="str">
-        <x:v>evt_001</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="115" ht="25" customHeight="1">
-      <x:c r="A115" s="3" t="str">
-        <x:v>Events</x:v>
-      </x:c>
-      <x:c r="B115" s="3" t="str">
-        <x:v>incident_002</x:v>
-      </x:c>
-      <x:c r="C115" s="3" t="str">
-        <x:v>Lost Caravan</x:v>
-      </x:c>
-      <x:c r="D115" s="3" t="str">
-        <x:v>Abandoned Delivery</x:v>
-      </x:c>
-      <x:c r="E115" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F115" s="3" t="str">
-        <x:v>Choice mechanics and outcomes unchanged</x:v>
-      </x:c>
-      <x:c r="G115" s="3" t="str">
-        <x:v>evt_002</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="116" ht="25" customHeight="1">
-      <x:c r="A116" s="3" t="str">
-        <x:v>Events</x:v>
-      </x:c>
-      <x:c r="B116" s="3" t="str">
-        <x:v>incident_003</x:v>
-      </x:c>
-      <x:c r="C116" s="3" t="str">
-        <x:v>Gambler's Shrine</x:v>
-      </x:c>
-      <x:c r="D116" s="3" t="str">
-        <x:v>Rigged Machine</x:v>
-      </x:c>
-      <x:c r="E116" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F116" s="3" t="str">
-        <x:v>Choice mechanics and outcomes unchanged</x:v>
-      </x:c>
-      <x:c r="G116" s="3" t="str">
-        <x:v>evt_003</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="117" ht="25" customHeight="1">
-      <x:c r="A117" s="3" t="str">
-        <x:v>Events</x:v>
-      </x:c>
-      <x:c r="B117" s="3" t="str">
-        <x:v>incident_004</x:v>
-      </x:c>
-      <x:c r="C117" s="3" t="str">
-        <x:v>Dangerous Shortcut</x:v>
-      </x:c>
-      <x:c r="D117" s="3" t="str">
-        <x:v>Service Tunnel</x:v>
-      </x:c>
-      <x:c r="E117" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F117" s="3" t="str">
-        <x:v>Choice mechanics and outcomes unchanged</x:v>
-      </x:c>
-      <x:c r="G117" s="3" t="str">
-        <x:v>evt_004</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="118" ht="25" customHeight="1">
-      <x:c r="A118" s="3" t="str">
-        <x:v>Events</x:v>
-      </x:c>
-      <x:c r="B118" s="3" t="str">
-        <x:v>incident_005</x:v>
-      </x:c>
-      <x:c r="C118" s="3" t="str">
-        <x:v>Blacksmith</x:v>
-      </x:c>
-      <x:c r="D118" s="3" t="str">
-        <x:v>Street Mechanic</x:v>
-      </x:c>
-      <x:c r="E118" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F118" s="3" t="str">
-        <x:v>Choice mechanics and outcomes unchanged</x:v>
-      </x:c>
-      <x:c r="G118" s="3" t="str">
-        <x:v>evt_005</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="119" ht="25" customHeight="1">
-      <x:c r="A119" s="3" t="str">
-        <x:v>Events</x:v>
-      </x:c>
-      <x:c r="B119" s="3" t="str">
-        <x:v>incident_006</x:v>
-      </x:c>
-      <x:c r="C119" s="3" t="str">
-        <x:v>Tavern</x:v>
-      </x:c>
-      <x:c r="D119" s="3" t="str">
-        <x:v>Late-Night Diner</x:v>
-      </x:c>
-      <x:c r="E119" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F119" s="3" t="str">
-        <x:v>Choice mechanics and outcomes unchanged</x:v>
-      </x:c>
-      <x:c r="G119" s="3" t="str">
-        <x:v>evt_006</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="120" ht="25" customHeight="1">
-      <x:c r="A120" s="3" t="str">
-        <x:v>Events</x:v>
-      </x:c>
-      <x:c r="B120" s="3" t="str">
-        <x:v>incident_007</x:v>
-      </x:c>
-      <x:c r="C120" s="3" t="str">
-        <x:v>Ambush</x:v>
-      </x:c>
-      <x:c r="D120" s="3" t="str">
-        <x:v>Back-Alley Trap</x:v>
-      </x:c>
-      <x:c r="E120" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F120" s="3" t="str">
-        <x:v>Choice mechanics and outcomes unchanged</x:v>
-      </x:c>
-      <x:c r="G120" s="3" t="str">
-        <x:v>evt_007</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="121" ht="25" customHeight="1">
-      <x:c r="A121" s="3" t="str">
-        <x:v>Events</x:v>
-      </x:c>
-      <x:c r="B121" s="3" t="str">
-        <x:v>incident_008</x:v>
-      </x:c>
-      <x:c r="C121" s="3" t="str">
-        <x:v>Mysterious Stranger</x:v>
-      </x:c>
-      <x:c r="D121" s="3" t="str">
-        <x:v>Anonymous Contact</x:v>
-      </x:c>
-      <x:c r="E121" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F121" s="3" t="str">
-        <x:v>Choice mechanics and outcomes unchanged</x:v>
-      </x:c>
-      <x:c r="G121" s="3" t="str">
-        <x:v>evt_008</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="122" ht="25" customHeight="1">
-      <x:c r="A122" s="3" t="str">
-        <x:v>Events</x:v>
-      </x:c>
-      <x:c r="B122" s="3" t="str">
-        <x:v>incident_009</x:v>
-      </x:c>
-      <x:c r="C122" s="3" t="str">
-        <x:v>Noble Family</x:v>
-      </x:c>
-      <x:c r="D122" s="3" t="str">
-        <x:v>VIP Party</x:v>
-      </x:c>
-      <x:c r="E122" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F122" s="3" t="str">
-        <x:v>Choice mechanics and outcomes unchanged</x:v>
-      </x:c>
-      <x:c r="G122" s="3" t="str">
-        <x:v>evt_009</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="123" ht="25" customHeight="1">
-      <x:c r="A123" s="3" t="str">
-        <x:v>Events</x:v>
-      </x:c>
-      <x:c r="B123" s="3" t="str">
-        <x:v>incident_010</x:v>
-      </x:c>
-      <x:c r="C123" s="3" t="str">
-        <x:v>Swamp</x:v>
-      </x:c>
-      <x:c r="D123" s="3" t="str">
-        <x:v>Toxic Runoff</x:v>
-      </x:c>
-      <x:c r="E123" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F123" s="3" t="str">
-        <x:v>Choice mechanics and outcomes unchanged</x:v>
-      </x:c>
-      <x:c r="G123" s="3" t="str">
-        <x:v>evt_010</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="124" ht="40" customHeight="1">
-      <x:c r="A124" s="3" t="str">
-        <x:v>Events</x:v>
-      </x:c>
-      <x:c r="B124" s="3" t="str">
-        <x:v>incident_100</x:v>
-      </x:c>
-      <x:c r="C124" s="3" t="str">
-        <x:v>Blood Ritual</x:v>
-      </x:c>
-      <x:c r="D124" s="3" t="str">
-        <x:v>Redline Deal</x:v>
-      </x:c>
-      <x:c r="E124" s="3" t="str">
-        <x:v>Implemented — awaiting phase acceptance</x:v>
-      </x:c>
-      <x:c r="F124" s="3" t="str">
-        <x:v>Choice mechanics and outcomes unchanged</x:v>
-      </x:c>
-      <x:c r="G124" s="3" t="str">
-        <x:v>evt_100</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="125" ht="25" customHeight="1">
-      <x:c r="A125" s="3" t="str">
-        <x:v>Events</x:v>
-      </x:c>
-      <x:c r="B125" s="3" t="str">
-        <x:v>incident_101</x:v>
-      </x:c>
-      <x:c r="C125" s="3" t="str">
-        <x:v>Field Lessons</x:v>
-      </x:c>
-      <x:c r="D125" s="3" t="str">
-        <x:v>Crash Course</x:v>
-      </x:c>
-      <x:c r="E125" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F125" s="3" t="str">
-        <x:v>Choice mechanics and outcomes unchanged</x:v>
-      </x:c>
-      <x:c r="G125" s="3" t="str">
-        <x:v>evt_101</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="126" ht="25" customHeight="1">
-      <x:c r="A126" s="3" t="str">
-        <x:v>Events</x:v>
-      </x:c>
-      <x:c r="B126" s="3" t="str">
-        <x:v>incident_102</x:v>
-      </x:c>
-      <x:c r="C126" s="3" t="str">
-        <x:v>Training Grounds</x:v>
-      </x:c>
-      <x:c r="D126" s="3" t="str">
-        <x:v>Test Lab</x:v>
-      </x:c>
-      <x:c r="E126" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F126" s="3" t="str">
-        <x:v>Choice mechanics and outcomes unchanged</x:v>
-      </x:c>
-      <x:c r="G126" s="3" t="str">
-        <x:v>evt_102</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="127" ht="25" customHeight="1">
-      <x:c r="A127" s="3" t="str">
-        <x:v>Shops</x:v>
-      </x:c>
-      <x:c r="B127" s="3" t="str">
-        <x:v>service_001</x:v>
-      </x:c>
-      <x:c r="C127" s="3" t="str">
-        <x:v>Investment</x:v>
-      </x:c>
-      <x:c r="D127" s="3" t="str">
-        <x:v>Stake</x:v>
-      </x:c>
-      <x:c r="E127" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F127" s="3" t="str">
-        <x:v>Service terms changed, effects unchanged</x:v>
-      </x:c>
-      <x:c r="G127" s="3" t="str">
-        <x:v>shop_001</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="128" ht="25" customHeight="1">
-      <x:c r="A128" s="3" t="str">
-        <x:v>Shops</x:v>
-      </x:c>
-      <x:c r="B128" s="3" t="str">
-        <x:v>service_002</x:v>
-      </x:c>
-      <x:c r="C128" s="3" t="str">
-        <x:v>Guidance</x:v>
-      </x:c>
-      <x:c r="D128" s="3" t="str">
-        <x:v>Intel</x:v>
-      </x:c>
-      <x:c r="E128" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F128" s="3" t="str">
-        <x:v>Service terms changed, effects unchanged</x:v>
-      </x:c>
-      <x:c r="G128" s="3" t="str">
-        <x:v>shop_002</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="129" ht="40" customHeight="1">
-      <x:c r="A129" s="3" t="str">
-        <x:v>Shops</x:v>
-      </x:c>
-      <x:c r="B129" s="3" t="str">
-        <x:v>service_003</x:v>
-      </x:c>
-      <x:c r="C129" s="3" t="str">
-        <x:v>Quest</x:v>
-      </x:c>
-      <x:c r="D129" s="3" t="str">
-        <x:v>Contract</x:v>
-      </x:c>
-      <x:c r="E129" s="3" t="str">
-        <x:v>Implemented — awaiting phase acceptance</x:v>
-      </x:c>
-      <x:c r="F129" s="3" t="str">
-        <x:v>Service terms changed, effects unchanged</x:v>
-      </x:c>
-      <x:c r="G129" s="3" t="str">
-        <x:v>shop_003</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="130" ht="25" customHeight="1">
-      <x:c r="A130" s="3" t="str">
-        <x:v>Maps</x:v>
-      </x:c>
-      <x:c r="B130" s="3" t="str">
-        <x:v>node_001</x:v>
-      </x:c>
-      <x:c r="C130" s="3" t="str">
-        <x:v>Normal Combat</x:v>
-      </x:c>
-      <x:c r="D130" s="3" t="str">
-        <x:v>Fight</x:v>
-      </x:c>
-      <x:c r="E130" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F130" s="3" t="str">
-        <x:v>Route mechanics unchanged</x:v>
-      </x:c>
-      <x:c r="G130" s="3"/>
-    </x:row>
-    <x:row r="131" ht="25" customHeight="1">
-      <x:c r="A131" s="3" t="str">
-        <x:v>Maps</x:v>
-      </x:c>
-      <x:c r="B131" s="3" t="str">
-        <x:v>node_002</x:v>
-      </x:c>
-      <x:c r="C131" s="3" t="str">
-        <x:v>Elite Combat</x:v>
-      </x:c>
-      <x:c r="D131" s="3" t="str">
-        <x:v>Enforcer</x:v>
-      </x:c>
-      <x:c r="E131" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F131" s="3" t="str">
-        <x:v>Route mechanics unchanged</x:v>
-      </x:c>
-      <x:c r="G131" s="3"/>
-    </x:row>
-    <x:row r="132" ht="25" customHeight="1">
-      <x:c r="A132" s="3" t="str">
-        <x:v>Maps</x:v>
-      </x:c>
-      <x:c r="B132" s="3" t="str">
-        <x:v>node_003</x:v>
-      </x:c>
-      <x:c r="C132" s="3" t="str">
-        <x:v>Boss Combat</x:v>
-      </x:c>
-      <x:c r="D132" s="3" t="str">
-        <x:v>Headliner</x:v>
-      </x:c>
-      <x:c r="E132" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F132" s="3" t="str">
-        <x:v>Route mechanics unchanged</x:v>
-      </x:c>
-      <x:c r="G132" s="3"/>
-    </x:row>
-    <x:row r="133" ht="25" customHeight="1">
-      <x:c r="A133" s="3" t="str">
-        <x:v>Maps</x:v>
-      </x:c>
-      <x:c r="B133" s="3" t="str">
-        <x:v>node_004</x:v>
-      </x:c>
-      <x:c r="C133" s="3" t="str">
-        <x:v>Shop</x:v>
-      </x:c>
-      <x:c r="D133" s="3" t="str">
-        <x:v>Black Market</x:v>
-      </x:c>
-      <x:c r="E133" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F133" s="3" t="str">
-        <x:v>Route mechanics unchanged</x:v>
-      </x:c>
-      <x:c r="G133" s="3"/>
-    </x:row>
-    <x:row r="134" ht="25" customHeight="1">
-      <x:c r="A134" s="3" t="str">
-        <x:v>Maps</x:v>
-      </x:c>
-      <x:c r="B134" s="3" t="str">
-        <x:v>node_005</x:v>
-      </x:c>
-      <x:c r="C134" s="3" t="str">
-        <x:v>Event</x:v>
-      </x:c>
-      <x:c r="D134" s="3" t="str">
-        <x:v>[Incident Name]</x:v>
-      </x:c>
-      <x:c r="E134" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F134" s="3" t="str">
-        <x:v>Route mechanics unchanged</x:v>
-      </x:c>
-      <x:c r="G134" s="3"/>
-    </x:row>
-    <x:row r="135" ht="25" customHeight="1">
-      <x:c r="A135" s="3" t="str">
-        <x:v>Consumables</x:v>
-      </x:c>
-      <x:c r="B135" s="3" t="str">
-        <x:v>consumable_001</x:v>
-      </x:c>
-      <x:c r="C135" s="3" t="str">
-        <x:v>Bread</x:v>
-      </x:c>
-      <x:c r="D135" s="3" t="str">
-        <x:v>Energy Bar</x:v>
-      </x:c>
-      <x:c r="E135" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F135" s="3" t="str">
-        <x:v>Same targets/charges and source</x:v>
-      </x:c>
-      <x:c r="G135" s="3" t="str">
-        <x:v>con_001</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="136" ht="25" customHeight="1">
-      <x:c r="A136" s="3" t="str">
-        <x:v>Consumables</x:v>
-      </x:c>
-      <x:c r="B136" s="3" t="str">
-        <x:v>consumable_002</x:v>
-      </x:c>
-      <x:c r="C136" s="3" t="str">
-        <x:v>Throwing Knife</x:v>
-      </x:c>
-      <x:c r="D136" s="3" t="str">
-        <x:v>Pocket Blade</x:v>
-      </x:c>
-      <x:c r="E136" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F136" s="3" t="str">
-        <x:v>Same targets/charges and source</x:v>
-      </x:c>
-      <x:c r="G136" s="3" t="str">
-        <x:v>con_002</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="137" ht="25" customHeight="1">
-      <x:c r="A137" s="3" t="str">
-        <x:v>Consumables</x:v>
-      </x:c>
-      <x:c r="B137" s="3" t="str">
-        <x:v>consumable_003</x:v>
-      </x:c>
-      <x:c r="C137" s="3" t="str">
-        <x:v>Whetstone</x:v>
-      </x:c>
-      <x:c r="D137" s="3" t="str">
-        <x:v>Power Patch</x:v>
-      </x:c>
-      <x:c r="E137" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F137" s="3" t="str">
-        <x:v>Same targets/charges and source</x:v>
-      </x:c>
-      <x:c r="G137" s="3" t="str">
-        <x:v>con_003</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="138" ht="25" customHeight="1">
-      <x:c r="A138" s="3" t="str">
-        <x:v>Consumables</x:v>
-      </x:c>
-      <x:c r="B138" s="3" t="str">
-        <x:v>consumable_004</x:v>
-      </x:c>
-      <x:c r="C138" s="3" t="str">
-        <x:v>Mirror</x:v>
-      </x:c>
-      <x:c r="D138" s="3" t="str">
-        <x:v>Copycat</x:v>
-      </x:c>
-      <x:c r="E138" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F138" s="3" t="str">
-        <x:v>Same targets/charges and source</x:v>
-      </x:c>
-      <x:c r="G138" s="3" t="str">
-        <x:v>con_004</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="139" ht="25" customHeight="1">
-      <x:c r="A139" s="3" t="str">
-        <x:v>Consumables</x:v>
-      </x:c>
-      <x:c r="B139" s="3" t="str">
-        <x:v>consumable_005</x:v>
-      </x:c>
-      <x:c r="C139" s="3" t="str">
-        <x:v>Torch</x:v>
-      </x:c>
-      <x:c r="D139" s="3" t="str">
-        <x:v>Shredder</x:v>
-      </x:c>
-      <x:c r="E139" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F139" s="3" t="str">
-        <x:v>Same targets/charges and source</x:v>
-      </x:c>
-      <x:c r="G139" s="3" t="str">
-        <x:v>con_005</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="140" ht="25" customHeight="1">
-      <x:c r="A140" s="3" t="str">
-        <x:v>Consumables</x:v>
-      </x:c>
-      <x:c r="B140" s="3" t="str">
-        <x:v>consumable_006</x:v>
-      </x:c>
-      <x:c r="C140" s="3" t="str">
-        <x:v>Bomb</x:v>
-      </x:c>
-      <x:c r="D140" s="3" t="str">
-        <x:v>Blast Patch</x:v>
-      </x:c>
-      <x:c r="E140" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F140" s="3" t="str">
-        <x:v>Same targets/charges and source</x:v>
-      </x:c>
-      <x:c r="G140" s="3" t="str">
-        <x:v>con_006</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="141" ht="25" customHeight="1">
-      <x:c r="A141" s="3" t="str">
-        <x:v>Consumables</x:v>
-      </x:c>
-      <x:c r="B141" s="3" t="str">
-        <x:v>consumable_007</x:v>
-      </x:c>
-      <x:c r="C141" s="3" t="str">
-        <x:v>Iron Plate</x:v>
-      </x:c>
-      <x:c r="D141" s="3" t="str">
-        <x:v>Armor Patch</x:v>
-      </x:c>
-      <x:c r="E141" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F141" s="3" t="str">
-        <x:v>Same targets/charges and source</x:v>
-      </x:c>
-      <x:c r="G141" s="3" t="str">
-        <x:v>con_007</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="142" ht="25" customHeight="1">
-      <x:c r="A142" s="3" t="str">
-        <x:v>Consumables</x:v>
-      </x:c>
-      <x:c r="B142" s="3" t="str">
-        <x:v>consumable_008</x:v>
-      </x:c>
-      <x:c r="C142" s="3" t="str">
-        <x:v>Needle &amp; Thread</x:v>
-      </x:c>
-      <x:c r="D142" s="3" t="str">
-        <x:v>Repair Patch</x:v>
-      </x:c>
-      <x:c r="E142" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F142" s="3" t="str">
-        <x:v>Same targets/charges and source</x:v>
-      </x:c>
-      <x:c r="G142" s="3" t="str">
-        <x:v>con_008</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="143" ht="25" customHeight="1">
-      <x:c r="A143" s="3" t="str">
-        <x:v>Consumables</x:v>
-      </x:c>
-      <x:c r="B143" s="3" t="str">
-        <x:v>consumable_009</x:v>
-      </x:c>
-      <x:c r="C143" s="3" t="str">
-        <x:v>Quiver</x:v>
-      </x:c>
-      <x:c r="D143" s="3" t="str">
-        <x:v>Draw Patch</x:v>
-      </x:c>
-      <x:c r="E143" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F143" s="3" t="str">
-        <x:v>Same targets/charges and source</x:v>
-      </x:c>
-      <x:c r="G143" s="3" t="str">
-        <x:v>con_009</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="144" ht="25" customHeight="1">
-      <x:c r="A144" s="3" t="str">
-        <x:v>Consumables</x:v>
-      </x:c>
-      <x:c r="B144" s="3" t="str">
-        <x:v>consumable_010</x:v>
-      </x:c>
-      <x:c r="C144" s="3" t="str">
-        <x:v>Soul Stone</x:v>
-      </x:c>
-      <x:c r="D144" s="3" t="str">
-        <x:v>Hunger Patch</x:v>
-      </x:c>
-      <x:c r="E144" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F144" s="3" t="str">
-        <x:v>Same targets/charges and source</x:v>
-      </x:c>
-      <x:c r="G144" s="3" t="str">
-        <x:v>con_010</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="145" ht="25" customHeight="1">
-      <x:c r="A145" s="3" t="str">
-        <x:v>Consumables</x:v>
-      </x:c>
-      <x:c r="B145" s="3" t="str">
-        <x:v>consumable_011</x:v>
-      </x:c>
-      <x:c r="C145" s="3" t="str">
-        <x:v>Venom</x:v>
-      </x:c>
-      <x:c r="D145" s="3" t="str">
-        <x:v>Crit Patch</x:v>
-      </x:c>
-      <x:c r="E145" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F145" s="3" t="str">
-        <x:v>Same targets/charges and source</x:v>
-      </x:c>
-      <x:c r="G145" s="3" t="str">
-        <x:v>con_011</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="146" ht="25" customHeight="1">
-      <x:c r="A146" s="3" t="str">
-        <x:v>Consumables</x:v>
-      </x:c>
-      <x:c r="B146" s="3" t="str">
-        <x:v>consumable_012</x:v>
-      </x:c>
-      <x:c r="C146" s="3" t="str">
-        <x:v>Midas Coin</x:v>
-      </x:c>
-      <x:c r="D146" s="3" t="str">
-        <x:v>Cash Patch</x:v>
-      </x:c>
-      <x:c r="E146" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F146" s="3" t="str">
-        <x:v>Same targets/charges and source</x:v>
-      </x:c>
-      <x:c r="G146" s="3" t="str">
-        <x:v>con_012</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="147" ht="25" customHeight="1">
-      <x:c r="A147" s="3" t="str">
-        <x:v>Consumables</x:v>
-      </x:c>
-      <x:c r="B147" s="3" t="str">
-        <x:v>consumable_013</x:v>
-      </x:c>
-      <x:c r="C147" s="3" t="str">
-        <x:v>Talisman</x:v>
-      </x:c>
-      <x:c r="D147" s="3" t="str">
-        <x:v>Support Patch</x:v>
-      </x:c>
-      <x:c r="E147" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F147" s="3" t="str">
-        <x:v>Same targets/charges and source</x:v>
-      </x:c>
-      <x:c r="G147" s="3" t="str">
-        <x:v>con_013</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="148" ht="25" customHeight="1">
-      <x:c r="A148" s="3" t="str">
-        <x:v>Consumables</x:v>
-      </x:c>
-      <x:c r="B148" s="3" t="str">
-        <x:v>consumable_014</x:v>
-      </x:c>
-      <x:c r="C148" s="3" t="str">
-        <x:v>Blood Vial</x:v>
-      </x:c>
-      <x:c r="D148" s="3" t="str">
-        <x:v>Overclock Patch</x:v>
-      </x:c>
-      <x:c r="E148" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F148" s="3" t="str">
-        <x:v>Same targets/charges and source</x:v>
-      </x:c>
-      <x:c r="G148" s="3" t="str">
-        <x:v>con_014</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="149" ht="25" customHeight="1">
-      <x:c r="A149" s="3" t="str">
-        <x:v>Consumables</x:v>
-      </x:c>
-      <x:c r="B149" s="3" t="str">
-        <x:v>consumable_015</x:v>
-      </x:c>
-      <x:c r="C149" s="3" t="str">
-        <x:v>Prism</x:v>
-      </x:c>
-      <x:c r="D149" s="3" t="str">
-        <x:v>Wild Patch</x:v>
-      </x:c>
-      <x:c r="E149" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F149" s="3" t="str">
-        <x:v>Same targets/charges and source</x:v>
-      </x:c>
-      <x:c r="G149" s="3" t="str">
-        <x:v>con_015</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="150" ht="25" customHeight="1">
-      <x:c r="A150" s="3" t="str">
-        <x:v>Consumables</x:v>
-      </x:c>
-      <x:c r="B150" s="3" t="str">
-        <x:v>consumable_016</x:v>
-      </x:c>
-      <x:c r="C150" s="3" t="str">
-        <x:v>Spade Rune</x:v>
-      </x:c>
-      <x:c r="D150" s="3" t="str">
-        <x:v>Spade Switch</x:v>
-      </x:c>
-      <x:c r="E150" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F150" s="3" t="str">
-        <x:v>Same targets/charges and source</x:v>
-      </x:c>
-      <x:c r="G150" s="3" t="str">
-        <x:v>con_016</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="151" ht="25" customHeight="1">
-      <x:c r="A151" s="3" t="str">
-        <x:v>Consumables</x:v>
-      </x:c>
-      <x:c r="B151" s="3" t="str">
-        <x:v>consumable_017</x:v>
-      </x:c>
-      <x:c r="C151" s="3" t="str">
-        <x:v>Heart Rune</x:v>
-      </x:c>
-      <x:c r="D151" s="3" t="str">
-        <x:v>Heart Switch</x:v>
-      </x:c>
-      <x:c r="E151" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F151" s="3" t="str">
-        <x:v>Same targets/charges and source</x:v>
-      </x:c>
-      <x:c r="G151" s="3" t="str">
-        <x:v>con_017</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="152" ht="25" customHeight="1">
-      <x:c r="A152" s="3" t="str">
-        <x:v>Consumables</x:v>
-      </x:c>
-      <x:c r="B152" s="3" t="str">
-        <x:v>consumable_018</x:v>
-      </x:c>
-      <x:c r="C152" s="3" t="str">
-        <x:v>Club Rune</x:v>
-      </x:c>
-      <x:c r="D152" s="3" t="str">
-        <x:v>Club Switch</x:v>
-      </x:c>
-      <x:c r="E152" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F152" s="3" t="str">
-        <x:v>Same targets/charges and source</x:v>
-      </x:c>
-      <x:c r="G152" s="3" t="str">
-        <x:v>con_018</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="153" ht="25" customHeight="1">
-      <x:c r="A153" s="3" t="str">
-        <x:v>Consumables</x:v>
-      </x:c>
-      <x:c r="B153" s="3" t="str">
-        <x:v>consumable_019</x:v>
-      </x:c>
-      <x:c r="C153" s="3" t="str">
-        <x:v>Diamond Rune</x:v>
-      </x:c>
-      <x:c r="D153" s="3" t="str">
-        <x:v>Diamond Switch</x:v>
-      </x:c>
-      <x:c r="E153" s="3" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="F153" s="3" t="str">
-        <x:v>Same targets/charges and source</x:v>
-      </x:c>
-      <x:c r="G153" s="3" t="str">
-        <x:v>con_019</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="154" ht="25" customHeight="1">
-      <x:c r="A154" s="3" t="str">
-        <x:v>Headliner Abilities</x:v>
-      </x:c>
-      <x:c r="B154" s="3" t="str">
-        <x:v>headliner_ability_silence</x:v>
-      </x:c>
-      <x:c r="C154" s="3" t="str">
-        <x:v>Silence</x:v>
-      </x:c>
-      <x:c r="D154" s="3" t="str">
-        <x:v>Signal Jam</x:v>
-      </x:c>
-      <x:c r="E154" s="3" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="F154" s="3" t="str">
-        <x:v>Same timing/threshold/mechanics</x:v>
-      </x:c>
-      <x:c r="G154" s="3" t="str">
-        <x:v>boss_ability_silence</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="155" ht="25" customHeight="1">
-      <x:c r="A155" s="3" t="str">
-        <x:v>Headliner Abilities</x:v>
-      </x:c>
-      <x:c r="B155" s="3" t="str">
-        <x:v>headliner_ability_wither</x:v>
-      </x:c>
-      <x:c r="C155" s="3" t="str">
-        <x:v>Withering</x:v>
-      </x:c>
-      <x:c r="D155" s="3" t="str">
-        <x:v>Heal Lock</x:v>
-      </x:c>
-      <x:c r="E155" s="3" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="F155" s="3" t="str">
-        <x:v>Same timing/threshold/mechanics</x:v>
-      </x:c>
-      <x:c r="G155" s="3" t="str">
-        <x:v>boss_ability_wither</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="156" ht="25" customHeight="1">
-      <x:c r="A156" s="3" t="str">
-        <x:v>Headliner Abilities</x:v>
-      </x:c>
-      <x:c r="B156" s="3" t="str">
-        <x:v>headliner_ability_oppression</x:v>
-      </x:c>
-      <x:c r="C156" s="3" t="str">
-        <x:v>Oppression</x:v>
-      </x:c>
-      <x:c r="D156" s="3" t="str">
-        <x:v>Pressure Tax</x:v>
-      </x:c>
-      <x:c r="E156" s="3" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="F156" s="3" t="str">
-        <x:v>Same timing/threshold/mechanics</x:v>
-      </x:c>
-      <x:c r="G156" s="3" t="str">
-        <x:v>boss_ability_oppression</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="157" ht="25" customHeight="1">
-      <x:c r="A157" s="3" t="str">
-        <x:v>Headliner Abilities</x:v>
-      </x:c>
-      <x:c r="B157" s="3" t="str">
-        <x:v>headliner_ability_regeneration</x:v>
-      </x:c>
-      <x:c r="C157" s="3" t="str">
-        <x:v>Regeneration</x:v>
-      </x:c>
-      <x:c r="D157" s="3" t="str">
-        <x:v>Self-Repair</x:v>
-      </x:c>
-      <x:c r="E157" s="3" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="F157" s="3" t="str">
-        <x:v>Same timing/threshold/mechanics</x:v>
-      </x:c>
-      <x:c r="G157" s="3" t="str">
-        <x:v>boss_ability_regeneration</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="158" ht="40" customHeight="1">
-      <x:c r="A158" s="3" t="str">
-        <x:v>Headliner Abilities</x:v>
-      </x:c>
-      <x:c r="B158" s="3" t="str">
-        <x:v>headliner_ability_double_strike</x:v>
-      </x:c>
-      <x:c r="C158" s="3" t="str">
-        <x:v>Double Strike</x:v>
-      </x:c>
-      <x:c r="D158" s="3" t="str">
-        <x:v>Double Tap</x:v>
-      </x:c>
-      <x:c r="E158" s="3" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="F158" s="3" t="str">
-        <x:v>Same timing/threshold/mechanics</x:v>
-      </x:c>
-      <x:c r="G158" s="3" t="str">
-        <x:v>boss_ability_double_strike</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="159" ht="25" customHeight="1">
-      <x:c r="A159" s="3" t="str">
-        <x:v>Headliner Abilities</x:v>
-      </x:c>
-      <x:c r="B159" s="3" t="str">
-        <x:v>headliner_ability_heavy_swing</x:v>
-      </x:c>
-      <x:c r="C159" s="3" t="str">
-        <x:v>Heavy Swing</x:v>
-      </x:c>
-      <x:c r="D159" s="3" t="str">
-        <x:v>Power Hit</x:v>
-      </x:c>
-      <x:c r="E159" s="3" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="F159" s="3" t="str">
-        <x:v>Same timing/threshold/mechanics</x:v>
-      </x:c>
-      <x:c r="G159" s="3" t="str">
-        <x:v>boss_ability_heavy_swing</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="160" ht="25" customHeight="1">
-      <x:c r="A160" s="3" t="str">
-        <x:v>Headliner Abilities</x:v>
-      </x:c>
-      <x:c r="B160" s="3" t="str">
-        <x:v>headliner_ability_guarded</x:v>
-      </x:c>
-      <x:c r="C160" s="3" t="str">
-        <x:v>Guarded</x:v>
-      </x:c>
-      <x:c r="D160" s="3" t="str">
-        <x:v>Guard Mode</x:v>
-      </x:c>
-      <x:c r="E160" s="3" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="F160" s="3" t="str">
-        <x:v>Same timing/threshold/mechanics</x:v>
-      </x:c>
-      <x:c r="G160" s="3" t="str">
-        <x:v>boss_ability_guarded</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="161" ht="25" customHeight="1">
-      <x:c r="A161" s="3" t="str">
-        <x:v>Headliner Abilities</x:v>
-      </x:c>
-      <x:c r="B161" s="3" t="str">
-        <x:v>headliner_ability_desperation</x:v>
-      </x:c>
-      <x:c r="C161" s="3" t="str">
-        <x:v>Desperation</x:v>
-      </x:c>
-      <x:c r="D161" s="3" t="str">
-        <x:v>Last Stand</x:v>
-      </x:c>
-      <x:c r="E161" s="3" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="F161" s="3" t="str">
-        <x:v>Same timing/threshold/mechanics</x:v>
-      </x:c>
-      <x:c r="G161" s="3" t="str">
-        <x:v>boss_ability_desperation</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="162" ht="40" customHeight="1">
-      <x:c r="A162" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B162" s="3" t="str">
-        <x:v>gear_035</x:v>
-      </x:c>
-      <x:c r="C162" s="3"/>
-      <x:c r="D162" s="3" t="str">
-        <x:v>Ghost Lens</x:v>
-      </x:c>
-      <x:c r="E162" s="3" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="F162" s="3" t="str">
-        <x:v>Named entry retained from Gear; legacy name and Unity ID not supplied.</x:v>
-      </x:c>
-      <x:c r="G162" s="3"/>
-    </x:row>
-    <x:row r="163" ht="40" customHeight="1">
-      <x:c r="A163" s="3" t="str">
-        <x:v>Gear</x:v>
-      </x:c>
-      <x:c r="B163" s="3" t="str">
-        <x:v>gear_036</x:v>
-      </x:c>
-      <x:c r="C163" s="3"/>
-      <x:c r="D163" s="3" t="str">
-        <x:v>Dealbreaker</x:v>
-      </x:c>
-      <x:c r="E163" s="3" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="F163" s="3" t="str">
-        <x:v>Named entry retained from Gear; legacy name and Unity ID not supplied.</x:v>
-      </x:c>
-      <x:c r="G163" s="3"/>
-    </x:row>
-  </x:sheetData>
-  <x:mergeCells>
-    <x:mergeCell ref="A1:F1"/>
-    <x:mergeCell ref="A2:F2"/>
-  </x:mergeCells>
-  <x:conditionalFormatting sqref="E5:E163">
-    <x:cfRule type="containsText" dxfId="20" priority="1" operator="containsText" text="Draft"/>
-    <x:cfRule type="containsText" dxfId="21" priority="2" operator="containsText" text="Rework"/>
-  </x:conditionalFormatting>
-  <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="E5:E163">
-      <x:formula1>"Idea,Draft,Approved,Implemented,Needs Rework,Cut,Implemented — awaiting phase acceptance,Deferred by owner — redundant visibility; not implemented"</x:formula1>
-    </x:dataValidation>
-  </x:dataValidations>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
 
@@ -6493,7 +2145,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbcd528367cc546d4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c362a8a10374129"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9961,7 +5613,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98949ae5e727437d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89011ca2b0e54888"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10512,7 +6164,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6138eee3238943a2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ca5318a9d9e4cc5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11108,7 +6760,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04d6a42c2b814bf6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94a98d98590342e2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11268,7 +6920,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R695c2185f39f4fe3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b5a5a4b1b014e9b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11483,7 +7135,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49d685c5a2d64e1f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2131daacae144072"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12197,7 +7849,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c5ad718cda14968"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7caac0d66c80490b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12488,7 +8140,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63080d06a6ec4852"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e69f7249c0748b2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>